<commit_message>
test(golden): rótulos manuais de 5 municípios x 19 critérios
</commit_message>
<xml_diff>
--- a/golden/golden_set.xlsx
+++ b/golden/golden_set.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Gerson\Documents\CASE MPRJ 2026\monitor-transparencia\golden\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1DC77E8E-CE09-4CB6-9AE0-35DA2EAAB469}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4D4D3994-31A8-45F5-BFC1-C9338603A85B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="14400" yWindow="0" windowWidth="14400" windowHeight="15600" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="rotulos" sheetId="1" r:id="rId1"/>
@@ -24,7 +24,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="887" uniqueCount="165">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="896" uniqueCount="166">
   <si>
     <t>entidade</t>
   </si>
@@ -551,6 +551,9 @@
   </si>
   <si>
     <t>transparencia.duquedecaxias.rj.gov.br/?serv=1473</t>
+  </si>
+  <si>
+    <t>Servidor Municipal – PORTAL DA TRANSPARÊNCIA RIO</t>
   </si>
 </sst>
 </file>
@@ -949,6 +952,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
+  <sheetPr filterMode="1"/>
   <dimension ref="A1:K96"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
@@ -999,7 +1003,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="2" spans="1:11" ht="45" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:11" ht="45" hidden="1" x14ac:dyDescent="0.25">
       <c r="A2" s="3" t="s">
         <v>11</v>
       </c>
@@ -1034,7 +1038,7 @@
         <v>46309</v>
       </c>
     </row>
-    <row r="3" spans="1:11" ht="90" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:11" ht="90" hidden="1" x14ac:dyDescent="0.25">
       <c r="A3" s="3" t="s">
         <v>11</v>
       </c>
@@ -1069,7 +1073,7 @@
         <v>46309</v>
       </c>
     </row>
-    <row r="4" spans="1:11" ht="45" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:11" ht="45" hidden="1" x14ac:dyDescent="0.25">
       <c r="A4" s="3" t="s">
         <v>11</v>
       </c>
@@ -1104,7 +1108,7 @@
         <v>46309</v>
       </c>
     </row>
-    <row r="5" spans="1:11" ht="60" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:11" ht="60" hidden="1" x14ac:dyDescent="0.25">
       <c r="A5" s="3" t="s">
         <v>11</v>
       </c>
@@ -1139,7 +1143,7 @@
         <v>46309</v>
       </c>
     </row>
-    <row r="6" spans="1:11" ht="75" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:11" ht="75" hidden="1" x14ac:dyDescent="0.25">
       <c r="A6" s="3" t="s">
         <v>11</v>
       </c>
@@ -1174,7 +1178,7 @@
         <v>46309</v>
       </c>
     </row>
-    <row r="7" spans="1:11" ht="90" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:11" ht="90" hidden="1" x14ac:dyDescent="0.25">
       <c r="A7" s="3" t="s">
         <v>11</v>
       </c>
@@ -1207,7 +1211,7 @@
         <v>46309</v>
       </c>
     </row>
-    <row r="8" spans="1:11" ht="90" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:11" ht="90" hidden="1" x14ac:dyDescent="0.25">
       <c r="A8" s="3" t="s">
         <v>11</v>
       </c>
@@ -1242,7 +1246,7 @@
         <v>46309</v>
       </c>
     </row>
-    <row r="9" spans="1:11" ht="75" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:11" ht="75" hidden="1" x14ac:dyDescent="0.25">
       <c r="A9" s="3" t="s">
         <v>11</v>
       </c>
@@ -1267,7 +1271,9 @@
       <c r="H9" s="3" t="s">
         <v>130</v>
       </c>
-      <c r="I9" s="3"/>
+      <c r="I9" s="5" t="s">
+        <v>165</v>
+      </c>
       <c r="J9" s="3" t="s">
         <v>131</v>
       </c>
@@ -1275,7 +1281,7 @@
         <v>46309</v>
       </c>
     </row>
-    <row r="10" spans="1:11" ht="90" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:11" ht="90" hidden="1" x14ac:dyDescent="0.25">
       <c r="A10" s="3" t="s">
         <v>11</v>
       </c>
@@ -1310,7 +1316,7 @@
         <v>46309</v>
       </c>
     </row>
-    <row r="11" spans="1:11" ht="60" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:11" ht="60" hidden="1" x14ac:dyDescent="0.25">
       <c r="A11" s="3" t="s">
         <v>11</v>
       </c>
@@ -1345,7 +1351,7 @@
         <v>46309</v>
       </c>
     </row>
-    <row r="12" spans="1:11" ht="120" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:11" ht="120" hidden="1" x14ac:dyDescent="0.25">
       <c r="A12" s="3" t="s">
         <v>11</v>
       </c>
@@ -1380,7 +1386,7 @@
         <v>46309</v>
       </c>
     </row>
-    <row r="13" spans="1:11" ht="45" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:11" ht="45" hidden="1" x14ac:dyDescent="0.25">
       <c r="A13" s="3" t="s">
         <v>11</v>
       </c>
@@ -1413,7 +1419,7 @@
         <v>46309</v>
       </c>
     </row>
-    <row r="14" spans="1:11" ht="60" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:11" ht="60" hidden="1" x14ac:dyDescent="0.25">
       <c r="A14" s="3" t="s">
         <v>11</v>
       </c>
@@ -1446,7 +1452,7 @@
         <v>46309</v>
       </c>
     </row>
-    <row r="15" spans="1:11" ht="75" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:11" ht="75" hidden="1" x14ac:dyDescent="0.25">
       <c r="A15" s="3" t="s">
         <v>11</v>
       </c>
@@ -1479,7 +1485,7 @@
         <v>46309</v>
       </c>
     </row>
-    <row r="16" spans="1:11" ht="90" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:11" ht="90" hidden="1" x14ac:dyDescent="0.25">
       <c r="A16" s="3" t="s">
         <v>11</v>
       </c>
@@ -1512,7 +1518,7 @@
         <v>46309</v>
       </c>
     </row>
-    <row r="17" spans="1:11" ht="90" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:11" ht="90" hidden="1" x14ac:dyDescent="0.25">
       <c r="A17" s="3" t="s">
         <v>11</v>
       </c>
@@ -1545,7 +1551,7 @@
         <v>46311</v>
       </c>
     </row>
-    <row r="18" spans="1:11" ht="60" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:11" ht="60" hidden="1" x14ac:dyDescent="0.25">
       <c r="A18" s="3" t="s">
         <v>11</v>
       </c>
@@ -1578,7 +1584,7 @@
         <v>46311</v>
       </c>
     </row>
-    <row r="19" spans="1:11" ht="60" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:11" ht="60" hidden="1" x14ac:dyDescent="0.25">
       <c r="A19" s="3" t="s">
         <v>11</v>
       </c>
@@ -1611,7 +1617,7 @@
         <v>46311</v>
       </c>
     </row>
-    <row r="20" spans="1:11" ht="105" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:11" ht="105" hidden="1" x14ac:dyDescent="0.25">
       <c r="A20" s="3" t="s">
         <v>11</v>
       </c>
@@ -1644,7 +1650,7 @@
         <v>46311</v>
       </c>
     </row>
-    <row r="21" spans="1:11" ht="45" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:11" ht="45" hidden="1" x14ac:dyDescent="0.25">
       <c r="A21" s="3" t="s">
         <v>89</v>
       </c>
@@ -1677,7 +1683,7 @@
         <v>46311</v>
       </c>
     </row>
-    <row r="22" spans="1:11" ht="90" x14ac:dyDescent="0.25">
+    <row r="22" spans="1:11" ht="90" hidden="1" x14ac:dyDescent="0.25">
       <c r="A22" s="3" t="s">
         <v>89</v>
       </c>
@@ -1710,7 +1716,7 @@
         <v>46311</v>
       </c>
     </row>
-    <row r="23" spans="1:11" ht="45" x14ac:dyDescent="0.25">
+    <row r="23" spans="1:11" ht="45" hidden="1" x14ac:dyDescent="0.25">
       <c r="A23" s="3" t="s">
         <v>89</v>
       </c>
@@ -1743,7 +1749,7 @@
         <v>46311</v>
       </c>
     </row>
-    <row r="24" spans="1:11" ht="60" x14ac:dyDescent="0.25">
+    <row r="24" spans="1:11" ht="60" hidden="1" x14ac:dyDescent="0.25">
       <c r="A24" s="3" t="s">
         <v>95</v>
       </c>
@@ -1776,7 +1782,7 @@
         <v>46311</v>
       </c>
     </row>
-    <row r="25" spans="1:11" ht="75" x14ac:dyDescent="0.25">
+    <row r="25" spans="1:11" ht="75" hidden="1" x14ac:dyDescent="0.25">
       <c r="A25" s="3" t="s">
         <v>89</v>
       </c>
@@ -1801,13 +1807,15 @@
       <c r="H25" s="3" t="s">
         <v>120</v>
       </c>
-      <c r="I25" s="3"/>
+      <c r="I25" s="3" t="s">
+        <v>91</v>
+      </c>
       <c r="J25" s="3"/>
       <c r="K25" s="6">
         <v>46311</v>
       </c>
     </row>
-    <row r="26" spans="1:11" ht="75" x14ac:dyDescent="0.25">
+    <row r="26" spans="1:11" ht="75" hidden="1" x14ac:dyDescent="0.25">
       <c r="A26" s="3" t="s">
         <v>92</v>
       </c>
@@ -1832,13 +1840,15 @@
       <c r="H26" s="3" t="s">
         <v>123</v>
       </c>
-      <c r="I26" s="3"/>
+      <c r="I26" s="3" t="s">
+        <v>94</v>
+      </c>
       <c r="J26" s="3"/>
       <c r="K26" s="6">
         <v>46311</v>
       </c>
     </row>
-    <row r="27" spans="1:11" ht="75" x14ac:dyDescent="0.25">
+    <row r="27" spans="1:11" ht="75" hidden="1" x14ac:dyDescent="0.25">
       <c r="A27" s="3" t="s">
         <v>95</v>
       </c>
@@ -1863,13 +1873,15 @@
       <c r="H27" s="3" t="s">
         <v>123</v>
       </c>
-      <c r="I27" s="3"/>
+      <c r="I27" s="3" t="s">
+        <v>97</v>
+      </c>
       <c r="J27" s="3"/>
       <c r="K27" s="6">
         <v>46311</v>
       </c>
     </row>
-    <row r="28" spans="1:11" ht="75" x14ac:dyDescent="0.25">
+    <row r="28" spans="1:11" ht="75" hidden="1" x14ac:dyDescent="0.25">
       <c r="A28" s="3" t="s">
         <v>98</v>
       </c>
@@ -1894,13 +1906,15 @@
       <c r="H28" s="3" t="s">
         <v>120</v>
       </c>
-      <c r="I28" s="3"/>
+      <c r="I28" s="3" t="s">
+        <v>99</v>
+      </c>
       <c r="J28" s="3"/>
       <c r="K28" s="6">
         <v>46311</v>
       </c>
     </row>
-    <row r="29" spans="1:11" ht="90" x14ac:dyDescent="0.25">
+    <row r="29" spans="1:11" ht="90" hidden="1" x14ac:dyDescent="0.25">
       <c r="A29" s="3" t="s">
         <v>89</v>
       </c>
@@ -1933,7 +1947,7 @@
         <v>46311</v>
       </c>
     </row>
-    <row r="30" spans="1:11" ht="60" x14ac:dyDescent="0.25">
+    <row r="30" spans="1:11" ht="60" hidden="1" x14ac:dyDescent="0.25">
       <c r="A30" s="3" t="s">
         <v>89</v>
       </c>
@@ -1966,7 +1980,7 @@
         <v>46311</v>
       </c>
     </row>
-    <row r="31" spans="1:11" ht="120" x14ac:dyDescent="0.25">
+    <row r="31" spans="1:11" ht="120" hidden="1" x14ac:dyDescent="0.25">
       <c r="A31" s="3" t="s">
         <v>89</v>
       </c>
@@ -1999,7 +2013,7 @@
         <v>46311</v>
       </c>
     </row>
-    <row r="32" spans="1:11" ht="45" x14ac:dyDescent="0.25">
+    <row r="32" spans="1:11" ht="45" hidden="1" x14ac:dyDescent="0.25">
       <c r="A32" s="3" t="s">
         <v>89</v>
       </c>
@@ -2032,7 +2046,7 @@
         <v>46311</v>
       </c>
     </row>
-    <row r="33" spans="1:11" ht="60" x14ac:dyDescent="0.25">
+    <row r="33" spans="1:11" ht="60" hidden="1" x14ac:dyDescent="0.25">
       <c r="A33" s="3" t="s">
         <v>89</v>
       </c>
@@ -2065,7 +2079,7 @@
         <v>46311</v>
       </c>
     </row>
-    <row r="34" spans="1:11" ht="90" x14ac:dyDescent="0.25">
+    <row r="34" spans="1:11" ht="90" hidden="1" x14ac:dyDescent="0.25">
       <c r="A34" s="3" t="s">
         <v>92</v>
       </c>
@@ -2098,7 +2112,7 @@
         <v>46311</v>
       </c>
     </row>
-    <row r="35" spans="1:11" ht="90" x14ac:dyDescent="0.25">
+    <row r="35" spans="1:11" ht="90" hidden="1" x14ac:dyDescent="0.25">
       <c r="A35" s="3" t="s">
         <v>95</v>
       </c>
@@ -2131,7 +2145,7 @@
         <v>46311</v>
       </c>
     </row>
-    <row r="36" spans="1:11" ht="90" x14ac:dyDescent="0.25">
+    <row r="36" spans="1:11" ht="90" hidden="1" x14ac:dyDescent="0.25">
       <c r="A36" s="3" t="s">
         <v>98</v>
       </c>
@@ -2164,7 +2178,7 @@
         <v>46311</v>
       </c>
     </row>
-    <row r="37" spans="1:11" ht="90" x14ac:dyDescent="0.25">
+    <row r="37" spans="1:11" ht="90" hidden="1" x14ac:dyDescent="0.25">
       <c r="A37" s="3" t="s">
         <v>89</v>
       </c>
@@ -2197,7 +2211,7 @@
         <v>46311</v>
       </c>
     </row>
-    <row r="38" spans="1:11" ht="90" x14ac:dyDescent="0.25">
+    <row r="38" spans="1:11" ht="90" hidden="1" x14ac:dyDescent="0.25">
       <c r="A38" s="3" t="s">
         <v>92</v>
       </c>
@@ -2230,7 +2244,7 @@
         <v>46311</v>
       </c>
     </row>
-    <row r="39" spans="1:11" ht="90" x14ac:dyDescent="0.25">
+    <row r="39" spans="1:11" ht="90" hidden="1" x14ac:dyDescent="0.25">
       <c r="A39" s="3" t="s">
         <v>95</v>
       </c>
@@ -2255,13 +2269,15 @@
       <c r="H39" s="3" t="s">
         <v>159</v>
       </c>
-      <c r="I39" s="5"/>
+      <c r="I39" s="5" t="s">
+        <v>145</v>
+      </c>
       <c r="J39" s="3"/>
       <c r="K39" s="6">
         <v>46311</v>
       </c>
     </row>
-    <row r="40" spans="1:11" ht="45" x14ac:dyDescent="0.25">
+    <row r="40" spans="1:11" ht="45" hidden="1" x14ac:dyDescent="0.25">
       <c r="A40" s="3" t="s">
         <v>92</v>
       </c>
@@ -2294,7 +2310,7 @@
         <v>46311</v>
       </c>
     </row>
-    <row r="41" spans="1:11" ht="90" x14ac:dyDescent="0.25">
+    <row r="41" spans="1:11" ht="90" hidden="1" x14ac:dyDescent="0.25">
       <c r="A41" s="3" t="s">
         <v>92</v>
       </c>
@@ -2327,7 +2343,7 @@
         <v>46311</v>
       </c>
     </row>
-    <row r="42" spans="1:11" ht="45" x14ac:dyDescent="0.25">
+    <row r="42" spans="1:11" ht="45" hidden="1" x14ac:dyDescent="0.25">
       <c r="A42" s="3" t="s">
         <v>92</v>
       </c>
@@ -2360,7 +2376,7 @@
         <v>46311</v>
       </c>
     </row>
-    <row r="43" spans="1:11" ht="90" x14ac:dyDescent="0.25">
+    <row r="43" spans="1:11" ht="90" hidden="1" x14ac:dyDescent="0.25">
       <c r="A43" s="3" t="s">
         <v>98</v>
       </c>
@@ -2393,7 +2409,7 @@
         <v>46311</v>
       </c>
     </row>
-    <row r="44" spans="1:11" ht="60" x14ac:dyDescent="0.25">
+    <row r="44" spans="1:11" ht="60" hidden="1" x14ac:dyDescent="0.25">
       <c r="A44" s="3" t="s">
         <v>89</v>
       </c>
@@ -2426,7 +2442,7 @@
         <v>46311</v>
       </c>
     </row>
-    <row r="45" spans="1:11" ht="60" x14ac:dyDescent="0.25">
+    <row r="45" spans="1:11" ht="60" hidden="1" x14ac:dyDescent="0.25">
       <c r="A45" s="3" t="s">
         <v>92</v>
       </c>
@@ -2459,7 +2475,7 @@
         <v>46311</v>
       </c>
     </row>
-    <row r="46" spans="1:11" ht="60" x14ac:dyDescent="0.25">
+    <row r="46" spans="1:11" ht="60" hidden="1" x14ac:dyDescent="0.25">
       <c r="A46" s="3" t="s">
         <v>95</v>
       </c>
@@ -2492,7 +2508,7 @@
         <v>46311</v>
       </c>
     </row>
-    <row r="47" spans="1:11" ht="60" x14ac:dyDescent="0.25">
+    <row r="47" spans="1:11" ht="60" hidden="1" x14ac:dyDescent="0.25">
       <c r="A47" s="3" t="s">
         <v>98</v>
       </c>
@@ -2525,7 +2541,7 @@
         <v>46311</v>
       </c>
     </row>
-    <row r="48" spans="1:11" ht="60" x14ac:dyDescent="0.25">
+    <row r="48" spans="1:11" ht="60" hidden="1" x14ac:dyDescent="0.25">
       <c r="A48" s="3" t="s">
         <v>89</v>
       </c>
@@ -2558,7 +2574,7 @@
         <v>46311</v>
       </c>
     </row>
-    <row r="49" spans="1:11" ht="60" x14ac:dyDescent="0.25">
+    <row r="49" spans="1:11" ht="60" hidden="1" x14ac:dyDescent="0.25">
       <c r="A49" s="3" t="s">
         <v>92</v>
       </c>
@@ -2616,13 +2632,15 @@
       <c r="H50" s="3" t="s">
         <v>130</v>
       </c>
-      <c r="I50" s="3"/>
+      <c r="I50" s="3" t="s">
+        <v>93</v>
+      </c>
       <c r="J50" s="3"/>
       <c r="K50" s="6">
         <v>46311</v>
       </c>
     </row>
-    <row r="51" spans="1:11" ht="45" x14ac:dyDescent="0.25">
+    <row r="51" spans="1:11" ht="45" hidden="1" x14ac:dyDescent="0.25">
       <c r="A51" s="3" t="s">
         <v>92</v>
       </c>
@@ -2655,7 +2673,7 @@
         <v>46311</v>
       </c>
     </row>
-    <row r="52" spans="1:11" ht="60" x14ac:dyDescent="0.25">
+    <row r="52" spans="1:11" ht="60" hidden="1" x14ac:dyDescent="0.25">
       <c r="A52" s="3" t="s">
         <v>92</v>
       </c>
@@ -2690,7 +2708,7 @@
         <v>46311</v>
       </c>
     </row>
-    <row r="53" spans="1:11" ht="60" x14ac:dyDescent="0.25">
+    <row r="53" spans="1:11" ht="60" hidden="1" x14ac:dyDescent="0.25">
       <c r="A53" s="3" t="s">
         <v>92</v>
       </c>
@@ -2723,7 +2741,7 @@
         <v>46311</v>
       </c>
     </row>
-    <row r="54" spans="1:11" ht="60" x14ac:dyDescent="0.25">
+    <row r="54" spans="1:11" ht="60" hidden="1" x14ac:dyDescent="0.25">
       <c r="A54" s="3" t="s">
         <v>95</v>
       </c>
@@ -2756,7 +2774,7 @@
         <v>46311</v>
       </c>
     </row>
-    <row r="55" spans="1:11" ht="60" x14ac:dyDescent="0.25">
+    <row r="55" spans="1:11" ht="60" hidden="1" x14ac:dyDescent="0.25">
       <c r="A55" s="3" t="s">
         <v>98</v>
       </c>
@@ -2789,7 +2807,7 @@
         <v>46311</v>
       </c>
     </row>
-    <row r="56" spans="1:11" ht="60" x14ac:dyDescent="0.25">
+    <row r="56" spans="1:11" ht="60" hidden="1" x14ac:dyDescent="0.25">
       <c r="A56" s="3" t="s">
         <v>89</v>
       </c>
@@ -2822,7 +2840,7 @@
         <v>46311</v>
       </c>
     </row>
-    <row r="57" spans="1:11" ht="60" x14ac:dyDescent="0.25">
+    <row r="57" spans="1:11" ht="60" hidden="1" x14ac:dyDescent="0.25">
       <c r="A57" s="3" t="s">
         <v>92</v>
       </c>
@@ -2855,7 +2873,7 @@
         <v>46311</v>
       </c>
     </row>
-    <row r="58" spans="1:11" ht="60" x14ac:dyDescent="0.25">
+    <row r="58" spans="1:11" ht="60" hidden="1" x14ac:dyDescent="0.25">
       <c r="A58" s="3" t="s">
         <v>95</v>
       </c>
@@ -2888,7 +2906,7 @@
         <v>46311</v>
       </c>
     </row>
-    <row r="59" spans="1:11" ht="45" x14ac:dyDescent="0.25">
+    <row r="59" spans="1:11" ht="45" hidden="1" x14ac:dyDescent="0.25">
       <c r="A59" s="3" t="s">
         <v>95</v>
       </c>
@@ -2921,7 +2939,7 @@
         <v>46311</v>
       </c>
     </row>
-    <row r="60" spans="1:11" ht="90" x14ac:dyDescent="0.25">
+    <row r="60" spans="1:11" ht="90" hidden="1" x14ac:dyDescent="0.25">
       <c r="A60" s="3" t="s">
         <v>95</v>
       </c>
@@ -2954,7 +2972,7 @@
         <v>46311</v>
       </c>
     </row>
-    <row r="61" spans="1:11" ht="45" x14ac:dyDescent="0.25">
+    <row r="61" spans="1:11" ht="45" hidden="1" x14ac:dyDescent="0.25">
       <c r="A61" s="3" t="s">
         <v>95</v>
       </c>
@@ -2987,7 +3005,7 @@
         <v>46311</v>
       </c>
     </row>
-    <row r="62" spans="1:11" ht="60" x14ac:dyDescent="0.25">
+    <row r="62" spans="1:11" ht="60" hidden="1" x14ac:dyDescent="0.25">
       <c r="A62" s="3" t="s">
         <v>98</v>
       </c>
@@ -3045,13 +3063,15 @@
       <c r="H63" s="3" t="s">
         <v>130</v>
       </c>
-      <c r="I63" s="3"/>
+      <c r="I63" s="3" t="s">
+        <v>91</v>
+      </c>
       <c r="J63" s="3"/>
       <c r="K63" s="6">
         <v>46311</v>
       </c>
     </row>
-    <row r="64" spans="1:11" ht="105" x14ac:dyDescent="0.25">
+    <row r="64" spans="1:11" ht="105" hidden="1" x14ac:dyDescent="0.25">
       <c r="A64" s="3" t="s">
         <v>92</v>
       </c>
@@ -3109,13 +3129,15 @@
       <c r="H65" s="3" t="s">
         <v>120</v>
       </c>
-      <c r="I65" s="3"/>
+      <c r="I65" s="3" t="s">
+        <v>97</v>
+      </c>
       <c r="J65" s="3"/>
       <c r="K65" s="6">
         <v>46311</v>
       </c>
     </row>
-    <row r="66" spans="1:11" ht="105" x14ac:dyDescent="0.25">
+    <row r="66" spans="1:11" ht="105" hidden="1" x14ac:dyDescent="0.25">
       <c r="A66" s="3" t="s">
         <v>98</v>
       </c>
@@ -3148,7 +3170,7 @@
         <v>46311</v>
       </c>
     </row>
-    <row r="67" spans="1:11" ht="75" x14ac:dyDescent="0.25">
+    <row r="67" spans="1:11" ht="75" hidden="1" x14ac:dyDescent="0.25">
       <c r="A67" s="3" t="s">
         <v>89</v>
       </c>
@@ -3181,7 +3203,7 @@
         <v>46311</v>
       </c>
     </row>
-    <row r="68" spans="1:11" ht="75" x14ac:dyDescent="0.25">
+    <row r="68" spans="1:11" ht="75" hidden="1" x14ac:dyDescent="0.25">
       <c r="A68" s="3" t="s">
         <v>92</v>
       </c>
@@ -3214,7 +3236,7 @@
         <v>46311</v>
       </c>
     </row>
-    <row r="69" spans="1:11" ht="120" x14ac:dyDescent="0.25">
+    <row r="69" spans="1:11" ht="120" hidden="1" x14ac:dyDescent="0.25">
       <c r="A69" s="3" t="s">
         <v>95</v>
       </c>
@@ -3247,7 +3269,7 @@
         <v>46311</v>
       </c>
     </row>
-    <row r="70" spans="1:11" ht="45" x14ac:dyDescent="0.25">
+    <row r="70" spans="1:11" ht="45" hidden="1" x14ac:dyDescent="0.25">
       <c r="A70" s="3" t="s">
         <v>95</v>
       </c>
@@ -3280,7 +3302,7 @@
         <v>46311</v>
       </c>
     </row>
-    <row r="71" spans="1:11" ht="60" x14ac:dyDescent="0.25">
+    <row r="71" spans="1:11" ht="60" hidden="1" x14ac:dyDescent="0.25">
       <c r="A71" s="3" t="s">
         <v>95</v>
       </c>
@@ -3313,7 +3335,7 @@
         <v>46311</v>
       </c>
     </row>
-    <row r="72" spans="1:11" ht="75" x14ac:dyDescent="0.25">
+    <row r="72" spans="1:11" ht="75" hidden="1" x14ac:dyDescent="0.25">
       <c r="A72" s="3" t="s">
         <v>95</v>
       </c>
@@ -3346,7 +3368,7 @@
         <v>46311</v>
       </c>
     </row>
-    <row r="73" spans="1:11" ht="75" x14ac:dyDescent="0.25">
+    <row r="73" spans="1:11" ht="75" hidden="1" x14ac:dyDescent="0.25">
       <c r="A73" s="3" t="s">
         <v>98</v>
       </c>
@@ -3379,7 +3401,7 @@
         <v>46311</v>
       </c>
     </row>
-    <row r="74" spans="1:11" ht="90" x14ac:dyDescent="0.25">
+    <row r="74" spans="1:11" ht="90" hidden="1" x14ac:dyDescent="0.25">
       <c r="A74" s="3" t="s">
         <v>89</v>
       </c>
@@ -3412,7 +3434,7 @@
         <v>46311</v>
       </c>
     </row>
-    <row r="75" spans="1:11" ht="90" x14ac:dyDescent="0.25">
+    <row r="75" spans="1:11" ht="90" hidden="1" x14ac:dyDescent="0.25">
       <c r="A75" s="3" t="s">
         <v>92</v>
       </c>
@@ -3445,7 +3467,7 @@
         <v>46311</v>
       </c>
     </row>
-    <row r="76" spans="1:11" ht="90" x14ac:dyDescent="0.25">
+    <row r="76" spans="1:11" ht="90" hidden="1" x14ac:dyDescent="0.25">
       <c r="A76" s="3" t="s">
         <v>95</v>
       </c>
@@ -3478,7 +3500,7 @@
         <v>46311</v>
       </c>
     </row>
-    <row r="77" spans="1:11" ht="90" x14ac:dyDescent="0.25">
+    <row r="77" spans="1:11" ht="90" hidden="1" x14ac:dyDescent="0.25">
       <c r="A77" s="3" t="s">
         <v>98</v>
       </c>
@@ -3511,7 +3533,7 @@
         <v>46311</v>
       </c>
     </row>
-    <row r="78" spans="1:11" ht="45" x14ac:dyDescent="0.25">
+    <row r="78" spans="1:11" ht="45" hidden="1" x14ac:dyDescent="0.25">
       <c r="A78" s="3" t="s">
         <v>98</v>
       </c>
@@ -3544,7 +3566,7 @@
         <v>46311</v>
       </c>
     </row>
-    <row r="79" spans="1:11" ht="90" x14ac:dyDescent="0.25">
+    <row r="79" spans="1:11" ht="90" hidden="1" x14ac:dyDescent="0.25">
       <c r="A79" s="3" t="s">
         <v>98</v>
       </c>
@@ -3577,7 +3599,7 @@
         <v>46311</v>
       </c>
     </row>
-    <row r="80" spans="1:11" ht="45" x14ac:dyDescent="0.25">
+    <row r="80" spans="1:11" ht="45" hidden="1" x14ac:dyDescent="0.25">
       <c r="A80" s="3" t="s">
         <v>98</v>
       </c>
@@ -3610,7 +3632,7 @@
         <v>46311</v>
       </c>
     </row>
-    <row r="81" spans="1:11" ht="90" x14ac:dyDescent="0.25">
+    <row r="81" spans="1:11" ht="90" hidden="1" x14ac:dyDescent="0.25">
       <c r="A81" s="3" t="s">
         <v>89</v>
       </c>
@@ -3643,7 +3665,7 @@
         <v>46311</v>
       </c>
     </row>
-    <row r="82" spans="1:11" ht="90" x14ac:dyDescent="0.25">
+    <row r="82" spans="1:11" ht="90" hidden="1" x14ac:dyDescent="0.25">
       <c r="A82" s="3" t="s">
         <v>92</v>
       </c>
@@ -3676,7 +3698,7 @@
         <v>46311</v>
       </c>
     </row>
-    <row r="83" spans="1:11" ht="90" x14ac:dyDescent="0.25">
+    <row r="83" spans="1:11" ht="90" hidden="1" x14ac:dyDescent="0.25">
       <c r="A83" s="3" t="s">
         <v>95</v>
       </c>
@@ -3709,7 +3731,7 @@
         <v>46311</v>
       </c>
     </row>
-    <row r="84" spans="1:11" ht="90" x14ac:dyDescent="0.25">
+    <row r="84" spans="1:11" ht="90" hidden="1" x14ac:dyDescent="0.25">
       <c r="A84" s="3" t="s">
         <v>98</v>
       </c>
@@ -3742,7 +3764,7 @@
         <v>46311</v>
       </c>
     </row>
-    <row r="85" spans="1:11" ht="75" x14ac:dyDescent="0.25">
+    <row r="85" spans="1:11" ht="75" hidden="1" x14ac:dyDescent="0.25">
       <c r="A85" s="3" t="s">
         <v>89</v>
       </c>
@@ -3775,7 +3797,7 @@
         <v>46311</v>
       </c>
     </row>
-    <row r="86" spans="1:11" ht="75" x14ac:dyDescent="0.25">
+    <row r="86" spans="1:11" ht="75" hidden="1" x14ac:dyDescent="0.25">
       <c r="A86" s="3" t="s">
         <v>92</v>
       </c>
@@ -3808,7 +3830,7 @@
         <v>46311</v>
       </c>
     </row>
-    <row r="87" spans="1:11" ht="60" x14ac:dyDescent="0.25">
+    <row r="87" spans="1:11" ht="60" hidden="1" x14ac:dyDescent="0.25">
       <c r="A87" s="3" t="s">
         <v>98</v>
       </c>
@@ -3841,7 +3863,7 @@
         <v>46311</v>
       </c>
     </row>
-    <row r="88" spans="1:11" ht="120" x14ac:dyDescent="0.25">
+    <row r="88" spans="1:11" ht="120" hidden="1" x14ac:dyDescent="0.25">
       <c r="A88" s="3" t="s">
         <v>98</v>
       </c>
@@ -3874,7 +3896,7 @@
         <v>46311</v>
       </c>
     </row>
-    <row r="89" spans="1:11" ht="45" x14ac:dyDescent="0.25">
+    <row r="89" spans="1:11" ht="45" hidden="1" x14ac:dyDescent="0.25">
       <c r="A89" s="3" t="s">
         <v>98</v>
       </c>
@@ -3907,7 +3929,7 @@
         <v>46311</v>
       </c>
     </row>
-    <row r="90" spans="1:11" ht="60" x14ac:dyDescent="0.25">
+    <row r="90" spans="1:11" ht="60" hidden="1" x14ac:dyDescent="0.25">
       <c r="A90" s="3" t="s">
         <v>98</v>
       </c>
@@ -3940,7 +3962,7 @@
         <v>46311</v>
       </c>
     </row>
-    <row r="91" spans="1:11" ht="75" x14ac:dyDescent="0.25">
+    <row r="91" spans="1:11" ht="75" hidden="1" x14ac:dyDescent="0.25">
       <c r="A91" s="3" t="s">
         <v>95</v>
       </c>
@@ -3973,7 +3995,7 @@
         <v>46311</v>
       </c>
     </row>
-    <row r="92" spans="1:11" ht="75" x14ac:dyDescent="0.25">
+    <row r="92" spans="1:11" ht="75" hidden="1" x14ac:dyDescent="0.25">
       <c r="A92" s="3" t="s">
         <v>98</v>
       </c>
@@ -4006,7 +4028,7 @@
         <v>46311</v>
       </c>
     </row>
-    <row r="93" spans="1:11" ht="90" x14ac:dyDescent="0.25">
+    <row r="93" spans="1:11" ht="90" hidden="1" x14ac:dyDescent="0.25">
       <c r="A93" s="3" t="s">
         <v>89</v>
       </c>
@@ -4039,7 +4061,7 @@
         <v>46311</v>
       </c>
     </row>
-    <row r="94" spans="1:11" ht="90" x14ac:dyDescent="0.25">
+    <row r="94" spans="1:11" ht="90" hidden="1" x14ac:dyDescent="0.25">
       <c r="A94" s="3" t="s">
         <v>92</v>
       </c>
@@ -4072,7 +4094,7 @@
         <v>46311</v>
       </c>
     </row>
-    <row r="95" spans="1:11" ht="90" x14ac:dyDescent="0.25">
+    <row r="95" spans="1:11" ht="90" hidden="1" x14ac:dyDescent="0.25">
       <c r="A95" s="3" t="s">
         <v>95</v>
       </c>
@@ -4105,7 +4127,7 @@
         <v>46311</v>
       </c>
     </row>
-    <row r="96" spans="1:11" ht="90" x14ac:dyDescent="0.25">
+    <row r="96" spans="1:11" ht="90" hidden="1" x14ac:dyDescent="0.25">
       <c r="A96" s="3" t="s">
         <v>98</v>
       </c>
@@ -4139,7 +4161,11 @@
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:K96" xr:uid="{00000000-0009-0000-0000-000000000000}"/>
+  <autoFilter ref="A1:K96" xr:uid="{00000000-0009-0000-0000-000000000000}">
+    <filterColumn colId="8">
+      <filters blank="1"/>
+    </filterColumn>
+  </autoFilter>
   <dataValidations count="1">
     <dataValidation type="list" allowBlank="1" error="Escolha um status da lista." sqref="H2:H37 H39:H96" xr:uid="{00000000-0002-0000-0000-000000000000}">
       <formula1>"ATENDE,ATENDE_PARCIALMENTE,NAO_ATENDE,NAO_SEI"</formula1>
@@ -4234,6 +4260,8 @@
     <hyperlink ref="I53" r:id="rId86" display="https://japeri.rj.gov.br/contato/" xr:uid="{EA0DB2E7-AA2A-4E14-A0F4-CA1612C1BF96}"/>
     <hyperlink ref="I55" r:id="rId87" display="https://falabr.cgu.gov.br/v2/" xr:uid="{AAF18F11-8D25-4476-920D-42DA5D55562E}"/>
     <hyperlink ref="I48" r:id="rId88" display="https://transparencia.duquedecaxias.rj.gov.br/?serv=1473" xr:uid="{93F38728-2763-4CF0-88C7-1EF465BF0B96}"/>
+    <hyperlink ref="I9" r:id="rId89" display="https://transparencia.prefeitura.rio/servidor-municipal/" xr:uid="{F3C8FF16-043F-4D3E-ADC7-989E4A4F4866}"/>
+    <hyperlink ref="I39" r:id="rId90" display="https://transparencianovo.ib.itaborai.rj.gov.br/" xr:uid="{817723A9-3570-487A-9170-3453AD1D7CF2}"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
test(golden): revisa 3 rótulos de Japeri divergentes da rubrica (15.2, 16.2, 16.3)
</commit_message>
<xml_diff>
--- a/golden/golden_set.xlsx
+++ b/golden/golden_set.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Gerson\Documents\CASE MPRJ 2026\monitor-transparencia\golden\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4D4D3994-31A8-45F5-BFC1-C9338603A85B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9E4145CC-3ACB-4671-9104-774211C210F0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="14400" yWindow="0" windowWidth="14400" windowHeight="15600" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -24,7 +24,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="896" uniqueCount="166">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="898" uniqueCount="167">
   <si>
     <t>entidade</t>
   </si>
@@ -520,9 +520,6 @@
     <t>Ouvidoria TRANSPARÊNCIA ITABORAÍ – Prefeitura Municipal de Itaboraí</t>
   </si>
   <si>
-    <t>apenas no site do portal da transparência</t>
-  </si>
-  <si>
     <t>LGPD – Prefeitura Municipal de Japeri</t>
   </si>
   <si>
@@ -554,6 +551,12 @@
   </si>
   <si>
     <t>Servidor Municipal – PORTAL DA TRANSPARÊNCIA RIO</t>
+  </si>
+  <si>
+    <t>revisada em 16/10/2026: identificado o icone de ouvidoria contendo o Fala.BR</t>
+  </si>
+  <si>
+    <t>revisada em 16/10/2026: identificado texto no topo da página</t>
   </si>
 </sst>
 </file>
@@ -629,7 +632,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="9">
+  <cellXfs count="10">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="1" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
@@ -649,6 +652,7 @@
     <xf numFmtId="14" fontId="4" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Hiperlink" xfId="1" builtinId="8"/>
@@ -952,8 +956,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <sheetPr filterMode="1"/>
-  <dimension ref="A1:K96"/>
+  <dimension ref="A1:N96"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="20" customWidth="1"/>
@@ -1003,7 +1006,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="2" spans="1:11" ht="45" hidden="1" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:11" ht="45" x14ac:dyDescent="0.25">
       <c r="A2" s="3" t="s">
         <v>11</v>
       </c>
@@ -1038,7 +1041,7 @@
         <v>46309</v>
       </c>
     </row>
-    <row r="3" spans="1:11" ht="90" hidden="1" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:11" ht="90" x14ac:dyDescent="0.25">
       <c r="A3" s="3" t="s">
         <v>11</v>
       </c>
@@ -1073,7 +1076,7 @@
         <v>46309</v>
       </c>
     </row>
-    <row r="4" spans="1:11" ht="45" hidden="1" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:11" ht="45" x14ac:dyDescent="0.25">
       <c r="A4" s="3" t="s">
         <v>11</v>
       </c>
@@ -1108,7 +1111,7 @@
         <v>46309</v>
       </c>
     </row>
-    <row r="5" spans="1:11" ht="60" hidden="1" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:11" ht="60" x14ac:dyDescent="0.25">
       <c r="A5" s="3" t="s">
         <v>11</v>
       </c>
@@ -1143,7 +1146,7 @@
         <v>46309</v>
       </c>
     </row>
-    <row r="6" spans="1:11" ht="75" hidden="1" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:11" ht="75" x14ac:dyDescent="0.25">
       <c r="A6" s="3" t="s">
         <v>11</v>
       </c>
@@ -1178,7 +1181,7 @@
         <v>46309</v>
       </c>
     </row>
-    <row r="7" spans="1:11" ht="90" hidden="1" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:11" ht="90" x14ac:dyDescent="0.25">
       <c r="A7" s="3" t="s">
         <v>11</v>
       </c>
@@ -1211,7 +1214,7 @@
         <v>46309</v>
       </c>
     </row>
-    <row r="8" spans="1:11" ht="90" hidden="1" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:11" ht="90" x14ac:dyDescent="0.25">
       <c r="A8" s="3" t="s">
         <v>11</v>
       </c>
@@ -1246,7 +1249,7 @@
         <v>46309</v>
       </c>
     </row>
-    <row r="9" spans="1:11" ht="75" hidden="1" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:11" ht="75" x14ac:dyDescent="0.25">
       <c r="A9" s="3" t="s">
         <v>11</v>
       </c>
@@ -1272,7 +1275,7 @@
         <v>130</v>
       </c>
       <c r="I9" s="5" t="s">
-        <v>165</v>
+        <v>164</v>
       </c>
       <c r="J9" s="3" t="s">
         <v>131</v>
@@ -1281,7 +1284,7 @@
         <v>46309</v>
       </c>
     </row>
-    <row r="10" spans="1:11" ht="90" hidden="1" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:11" ht="90" x14ac:dyDescent="0.25">
       <c r="A10" s="3" t="s">
         <v>11</v>
       </c>
@@ -1316,7 +1319,7 @@
         <v>46309</v>
       </c>
     </row>
-    <row r="11" spans="1:11" ht="60" hidden="1" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:11" ht="60" x14ac:dyDescent="0.25">
       <c r="A11" s="3" t="s">
         <v>11</v>
       </c>
@@ -1351,7 +1354,7 @@
         <v>46309</v>
       </c>
     </row>
-    <row r="12" spans="1:11" ht="120" hidden="1" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:11" ht="120" x14ac:dyDescent="0.25">
       <c r="A12" s="3" t="s">
         <v>11</v>
       </c>
@@ -1386,7 +1389,7 @@
         <v>46309</v>
       </c>
     </row>
-    <row r="13" spans="1:11" ht="45" hidden="1" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:11" ht="45" x14ac:dyDescent="0.25">
       <c r="A13" s="3" t="s">
         <v>11</v>
       </c>
@@ -1419,7 +1422,7 @@
         <v>46309</v>
       </c>
     </row>
-    <row r="14" spans="1:11" ht="60" hidden="1" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:11" ht="60" x14ac:dyDescent="0.25">
       <c r="A14" s="3" t="s">
         <v>11</v>
       </c>
@@ -1452,7 +1455,7 @@
         <v>46309</v>
       </c>
     </row>
-    <row r="15" spans="1:11" ht="75" hidden="1" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:11" ht="75" x14ac:dyDescent="0.25">
       <c r="A15" s="3" t="s">
         <v>11</v>
       </c>
@@ -1485,7 +1488,7 @@
         <v>46309</v>
       </c>
     </row>
-    <row r="16" spans="1:11" ht="90" hidden="1" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:11" ht="90" x14ac:dyDescent="0.25">
       <c r="A16" s="3" t="s">
         <v>11</v>
       </c>
@@ -1518,7 +1521,7 @@
         <v>46309</v>
       </c>
     </row>
-    <row r="17" spans="1:11" ht="90" hidden="1" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:11" ht="90" x14ac:dyDescent="0.25">
       <c r="A17" s="3" t="s">
         <v>11</v>
       </c>
@@ -1551,7 +1554,7 @@
         <v>46311</v>
       </c>
     </row>
-    <row r="18" spans="1:11" ht="60" hidden="1" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:11" ht="60" x14ac:dyDescent="0.25">
       <c r="A18" s="3" t="s">
         <v>11</v>
       </c>
@@ -1584,7 +1587,7 @@
         <v>46311</v>
       </c>
     </row>
-    <row r="19" spans="1:11" ht="60" hidden="1" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:11" ht="60" x14ac:dyDescent="0.25">
       <c r="A19" s="3" t="s">
         <v>11</v>
       </c>
@@ -1617,7 +1620,7 @@
         <v>46311</v>
       </c>
     </row>
-    <row r="20" spans="1:11" ht="105" hidden="1" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:11" ht="105" x14ac:dyDescent="0.25">
       <c r="A20" s="3" t="s">
         <v>11</v>
       </c>
@@ -1650,7 +1653,7 @@
         <v>46311</v>
       </c>
     </row>
-    <row r="21" spans="1:11" ht="45" hidden="1" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:11" ht="45" x14ac:dyDescent="0.25">
       <c r="A21" s="3" t="s">
         <v>89</v>
       </c>
@@ -1683,7 +1686,7 @@
         <v>46311</v>
       </c>
     </row>
-    <row r="22" spans="1:11" ht="90" hidden="1" x14ac:dyDescent="0.25">
+    <row r="22" spans="1:11" ht="90" x14ac:dyDescent="0.25">
       <c r="A22" s="3" t="s">
         <v>89</v>
       </c>
@@ -1716,7 +1719,7 @@
         <v>46311</v>
       </c>
     </row>
-    <row r="23" spans="1:11" ht="45" hidden="1" x14ac:dyDescent="0.25">
+    <row r="23" spans="1:11" ht="45" x14ac:dyDescent="0.25">
       <c r="A23" s="3" t="s">
         <v>89</v>
       </c>
@@ -1749,7 +1752,7 @@
         <v>46311</v>
       </c>
     </row>
-    <row r="24" spans="1:11" ht="60" hidden="1" x14ac:dyDescent="0.25">
+    <row r="24" spans="1:11" ht="60" x14ac:dyDescent="0.25">
       <c r="A24" s="3" t="s">
         <v>95</v>
       </c>
@@ -1782,7 +1785,7 @@
         <v>46311</v>
       </c>
     </row>
-    <row r="25" spans="1:11" ht="75" hidden="1" x14ac:dyDescent="0.25">
+    <row r="25" spans="1:11" ht="75" x14ac:dyDescent="0.25">
       <c r="A25" s="3" t="s">
         <v>89</v>
       </c>
@@ -1815,7 +1818,7 @@
         <v>46311</v>
       </c>
     </row>
-    <row r="26" spans="1:11" ht="75" hidden="1" x14ac:dyDescent="0.25">
+    <row r="26" spans="1:11" ht="75" x14ac:dyDescent="0.25">
       <c r="A26" s="3" t="s">
         <v>92</v>
       </c>
@@ -1848,7 +1851,7 @@
         <v>46311</v>
       </c>
     </row>
-    <row r="27" spans="1:11" ht="75" hidden="1" x14ac:dyDescent="0.25">
+    <row r="27" spans="1:11" ht="75" x14ac:dyDescent="0.25">
       <c r="A27" s="3" t="s">
         <v>95</v>
       </c>
@@ -1881,7 +1884,7 @@
         <v>46311</v>
       </c>
     </row>
-    <row r="28" spans="1:11" ht="75" hidden="1" x14ac:dyDescent="0.25">
+    <row r="28" spans="1:11" ht="75" x14ac:dyDescent="0.25">
       <c r="A28" s="3" t="s">
         <v>98</v>
       </c>
@@ -1914,7 +1917,7 @@
         <v>46311</v>
       </c>
     </row>
-    <row r="29" spans="1:11" ht="90" hidden="1" x14ac:dyDescent="0.25">
+    <row r="29" spans="1:11" ht="90" x14ac:dyDescent="0.25">
       <c r="A29" s="3" t="s">
         <v>89</v>
       </c>
@@ -1947,7 +1950,7 @@
         <v>46311</v>
       </c>
     </row>
-    <row r="30" spans="1:11" ht="60" hidden="1" x14ac:dyDescent="0.25">
+    <row r="30" spans="1:11" ht="60" x14ac:dyDescent="0.25">
       <c r="A30" s="3" t="s">
         <v>89</v>
       </c>
@@ -1980,7 +1983,7 @@
         <v>46311</v>
       </c>
     </row>
-    <row r="31" spans="1:11" ht="120" hidden="1" x14ac:dyDescent="0.25">
+    <row r="31" spans="1:11" ht="120" x14ac:dyDescent="0.25">
       <c r="A31" s="3" t="s">
         <v>89</v>
       </c>
@@ -2013,7 +2016,7 @@
         <v>46311</v>
       </c>
     </row>
-    <row r="32" spans="1:11" ht="45" hidden="1" x14ac:dyDescent="0.25">
+    <row r="32" spans="1:11" ht="45" x14ac:dyDescent="0.25">
       <c r="A32" s="3" t="s">
         <v>89</v>
       </c>
@@ -2046,7 +2049,7 @@
         <v>46311</v>
       </c>
     </row>
-    <row r="33" spans="1:11" ht="60" hidden="1" x14ac:dyDescent="0.25">
+    <row r="33" spans="1:11" ht="60" x14ac:dyDescent="0.25">
       <c r="A33" s="3" t="s">
         <v>89</v>
       </c>
@@ -2079,7 +2082,7 @@
         <v>46311</v>
       </c>
     </row>
-    <row r="34" spans="1:11" ht="90" hidden="1" x14ac:dyDescent="0.25">
+    <row r="34" spans="1:11" ht="90" x14ac:dyDescent="0.25">
       <c r="A34" s="3" t="s">
         <v>92</v>
       </c>
@@ -2105,14 +2108,14 @@
         <v>120</v>
       </c>
       <c r="I34" s="5" t="s">
-        <v>155</v>
+        <v>154</v>
       </c>
       <c r="J34" s="3"/>
       <c r="K34" s="6">
         <v>46311</v>
       </c>
     </row>
-    <row r="35" spans="1:11" ht="90" hidden="1" x14ac:dyDescent="0.25">
+    <row r="35" spans="1:11" ht="90" x14ac:dyDescent="0.25">
       <c r="A35" s="3" t="s">
         <v>95</v>
       </c>
@@ -2138,14 +2141,14 @@
         <v>120</v>
       </c>
       <c r="I35" s="5" t="s">
-        <v>156</v>
+        <v>155</v>
       </c>
       <c r="J35" s="3"/>
       <c r="K35" s="6">
         <v>46311</v>
       </c>
     </row>
-    <row r="36" spans="1:11" ht="90" hidden="1" x14ac:dyDescent="0.25">
+    <row r="36" spans="1:11" ht="90" x14ac:dyDescent="0.25">
       <c r="A36" s="3" t="s">
         <v>98</v>
       </c>
@@ -2178,7 +2181,7 @@
         <v>46311</v>
       </c>
     </row>
-    <row r="37" spans="1:11" ht="90" hidden="1" x14ac:dyDescent="0.25">
+    <row r="37" spans="1:11" ht="90" x14ac:dyDescent="0.25">
       <c r="A37" s="3" t="s">
         <v>89</v>
       </c>
@@ -2211,7 +2214,7 @@
         <v>46311</v>
       </c>
     </row>
-    <row r="38" spans="1:11" ht="90" hidden="1" x14ac:dyDescent="0.25">
+    <row r="38" spans="1:11" ht="90" x14ac:dyDescent="0.25">
       <c r="A38" s="3" t="s">
         <v>92</v>
       </c>
@@ -2244,7 +2247,7 @@
         <v>46311</v>
       </c>
     </row>
-    <row r="39" spans="1:11" ht="90" hidden="1" x14ac:dyDescent="0.25">
+    <row r="39" spans="1:11" ht="90" x14ac:dyDescent="0.25">
       <c r="A39" s="3" t="s">
         <v>95</v>
       </c>
@@ -2267,7 +2270,7 @@
         <v>97</v>
       </c>
       <c r="H39" s="3" t="s">
-        <v>159</v>
+        <v>158</v>
       </c>
       <c r="I39" s="5" t="s">
         <v>145</v>
@@ -2277,7 +2280,7 @@
         <v>46311</v>
       </c>
     </row>
-    <row r="40" spans="1:11" ht="45" hidden="1" x14ac:dyDescent="0.25">
+    <row r="40" spans="1:11" ht="45" x14ac:dyDescent="0.25">
       <c r="A40" s="3" t="s">
         <v>92</v>
       </c>
@@ -2310,7 +2313,7 @@
         <v>46311</v>
       </c>
     </row>
-    <row r="41" spans="1:11" ht="90" hidden="1" x14ac:dyDescent="0.25">
+    <row r="41" spans="1:11" ht="90" x14ac:dyDescent="0.25">
       <c r="A41" s="3" t="s">
         <v>92</v>
       </c>
@@ -2343,7 +2346,7 @@
         <v>46311</v>
       </c>
     </row>
-    <row r="42" spans="1:11" ht="45" hidden="1" x14ac:dyDescent="0.25">
+    <row r="42" spans="1:11" ht="45" x14ac:dyDescent="0.25">
       <c r="A42" s="3" t="s">
         <v>92</v>
       </c>
@@ -2376,7 +2379,7 @@
         <v>46311</v>
       </c>
     </row>
-    <row r="43" spans="1:11" ht="90" hidden="1" x14ac:dyDescent="0.25">
+    <row r="43" spans="1:11" ht="90" x14ac:dyDescent="0.25">
       <c r="A43" s="3" t="s">
         <v>98</v>
       </c>
@@ -2409,7 +2412,7 @@
         <v>46311</v>
       </c>
     </row>
-    <row r="44" spans="1:11" ht="60" hidden="1" x14ac:dyDescent="0.25">
+    <row r="44" spans="1:11" ht="60" x14ac:dyDescent="0.25">
       <c r="A44" s="3" t="s">
         <v>89</v>
       </c>
@@ -2442,7 +2445,7 @@
         <v>46311</v>
       </c>
     </row>
-    <row r="45" spans="1:11" ht="60" hidden="1" x14ac:dyDescent="0.25">
+    <row r="45" spans="1:11" ht="60" x14ac:dyDescent="0.25">
       <c r="A45" s="3" t="s">
         <v>92</v>
       </c>
@@ -2475,7 +2478,7 @@
         <v>46311</v>
       </c>
     </row>
-    <row r="46" spans="1:11" ht="60" hidden="1" x14ac:dyDescent="0.25">
+    <row r="46" spans="1:11" ht="60" x14ac:dyDescent="0.25">
       <c r="A46" s="3" t="s">
         <v>95</v>
       </c>
@@ -2501,14 +2504,14 @@
         <v>120</v>
       </c>
       <c r="I46" s="5" t="s">
-        <v>160</v>
+        <v>159</v>
       </c>
       <c r="J46" s="3"/>
       <c r="K46" s="6">
         <v>46311</v>
       </c>
     </row>
-    <row r="47" spans="1:11" ht="60" hidden="1" x14ac:dyDescent="0.25">
+    <row r="47" spans="1:11" ht="60" x14ac:dyDescent="0.25">
       <c r="A47" s="3" t="s">
         <v>98</v>
       </c>
@@ -2541,7 +2544,7 @@
         <v>46311</v>
       </c>
     </row>
-    <row r="48" spans="1:11" ht="60" hidden="1" x14ac:dyDescent="0.25">
+    <row r="48" spans="1:11" ht="60" x14ac:dyDescent="0.25">
       <c r="A48" s="3" t="s">
         <v>89</v>
       </c>
@@ -2567,14 +2570,14 @@
         <v>120</v>
       </c>
       <c r="I48" s="5" t="s">
-        <v>164</v>
+        <v>163</v>
       </c>
       <c r="J48" s="3"/>
       <c r="K48" s="6">
         <v>46311</v>
       </c>
     </row>
-    <row r="49" spans="1:11" ht="60" hidden="1" x14ac:dyDescent="0.25">
+    <row r="49" spans="1:14" ht="60" x14ac:dyDescent="0.25">
       <c r="A49" s="3" t="s">
         <v>92</v>
       </c>
@@ -2607,7 +2610,7 @@
         <v>46311</v>
       </c>
     </row>
-    <row r="50" spans="1:11" ht="120" x14ac:dyDescent="0.25">
+    <row r="50" spans="1:14" ht="120" x14ac:dyDescent="0.25">
       <c r="A50" s="3" t="s">
         <v>92</v>
       </c>
@@ -2630,17 +2633,19 @@
         <v>94</v>
       </c>
       <c r="H50" s="3" t="s">
-        <v>130</v>
-      </c>
-      <c r="I50" s="3" t="s">
-        <v>93</v>
-      </c>
-      <c r="J50" s="3"/>
+        <v>120</v>
+      </c>
+      <c r="I50" s="5" t="s">
+        <v>162</v>
+      </c>
+      <c r="J50" s="3" t="s">
+        <v>165</v>
+      </c>
       <c r="K50" s="6">
         <v>46311</v>
       </c>
     </row>
-    <row r="51" spans="1:11" ht="45" hidden="1" x14ac:dyDescent="0.25">
+    <row r="51" spans="1:14" ht="45" x14ac:dyDescent="0.25">
       <c r="A51" s="3" t="s">
         <v>92</v>
       </c>
@@ -2663,17 +2668,19 @@
         <v>94</v>
       </c>
       <c r="H51" s="3" t="s">
-        <v>130</v>
+        <v>120</v>
       </c>
       <c r="I51" s="5" t="s">
-        <v>148</v>
-      </c>
-      <c r="J51" s="3"/>
+        <v>144</v>
+      </c>
+      <c r="J51" s="3" t="s">
+        <v>166</v>
+      </c>
       <c r="K51" s="6">
         <v>46311</v>
       </c>
     </row>
-    <row r="52" spans="1:11" ht="60" hidden="1" x14ac:dyDescent="0.25">
+    <row r="52" spans="1:14" ht="60" x14ac:dyDescent="0.25">
       <c r="A52" s="3" t="s">
         <v>92</v>
       </c>
@@ -2696,19 +2703,20 @@
         <v>94</v>
       </c>
       <c r="H52" s="3" t="s">
-        <v>123</v>
-      </c>
-      <c r="I52" s="3" t="s">
-        <v>94</v>
+        <v>120</v>
+      </c>
+      <c r="I52" s="5" t="s">
+        <v>144</v>
       </c>
       <c r="J52" s="3" t="s">
-        <v>154</v>
+        <v>166</v>
       </c>
       <c r="K52" s="6">
         <v>46311</v>
       </c>
-    </row>
-    <row r="53" spans="1:11" ht="60" hidden="1" x14ac:dyDescent="0.25">
+      <c r="N52" s="9"/>
+    </row>
+    <row r="53" spans="1:14" ht="60" x14ac:dyDescent="0.25">
       <c r="A53" s="3" t="s">
         <v>92</v>
       </c>
@@ -2734,14 +2742,14 @@
         <v>120</v>
       </c>
       <c r="I53" s="5" t="s">
-        <v>162</v>
+        <v>161</v>
       </c>
       <c r="J53" s="3"/>
       <c r="K53" s="6">
         <v>46311</v>
       </c>
     </row>
-    <row r="54" spans="1:11" ht="60" hidden="1" x14ac:dyDescent="0.25">
+    <row r="54" spans="1:14" ht="60" x14ac:dyDescent="0.25">
       <c r="A54" s="3" t="s">
         <v>95</v>
       </c>
@@ -2774,7 +2782,7 @@
         <v>46311</v>
       </c>
     </row>
-    <row r="55" spans="1:11" ht="60" hidden="1" x14ac:dyDescent="0.25">
+    <row r="55" spans="1:14" ht="60" x14ac:dyDescent="0.25">
       <c r="A55" s="3" t="s">
         <v>98</v>
       </c>
@@ -2800,14 +2808,14 @@
         <v>120</v>
       </c>
       <c r="I55" s="5" t="s">
-        <v>163</v>
+        <v>162</v>
       </c>
       <c r="J55" s="3"/>
       <c r="K55" s="6">
         <v>46311</v>
       </c>
     </row>
-    <row r="56" spans="1:11" ht="60" hidden="1" x14ac:dyDescent="0.25">
+    <row r="56" spans="1:14" ht="60" x14ac:dyDescent="0.25">
       <c r="A56" s="3" t="s">
         <v>89</v>
       </c>
@@ -2840,7 +2848,7 @@
         <v>46311</v>
       </c>
     </row>
-    <row r="57" spans="1:11" ht="60" hidden="1" x14ac:dyDescent="0.25">
+    <row r="57" spans="1:14" ht="60" x14ac:dyDescent="0.25">
       <c r="A57" s="3" t="s">
         <v>92</v>
       </c>
@@ -2873,7 +2881,7 @@
         <v>46311</v>
       </c>
     </row>
-    <row r="58" spans="1:11" ht="60" hidden="1" x14ac:dyDescent="0.25">
+    <row r="58" spans="1:14" ht="60" x14ac:dyDescent="0.25">
       <c r="A58" s="3" t="s">
         <v>95</v>
       </c>
@@ -2899,14 +2907,14 @@
         <v>120</v>
       </c>
       <c r="I58" s="5" t="s">
-        <v>161</v>
+        <v>160</v>
       </c>
       <c r="J58" s="3"/>
       <c r="K58" s="6">
         <v>46311</v>
       </c>
     </row>
-    <row r="59" spans="1:11" ht="45" hidden="1" x14ac:dyDescent="0.25">
+    <row r="59" spans="1:14" ht="45" x14ac:dyDescent="0.25">
       <c r="A59" s="3" t="s">
         <v>95</v>
       </c>
@@ -2939,7 +2947,7 @@
         <v>46311</v>
       </c>
     </row>
-    <row r="60" spans="1:11" ht="90" hidden="1" x14ac:dyDescent="0.25">
+    <row r="60" spans="1:14" ht="90" x14ac:dyDescent="0.25">
       <c r="A60" s="3" t="s">
         <v>95</v>
       </c>
@@ -2972,7 +2980,7 @@
         <v>46311</v>
       </c>
     </row>
-    <row r="61" spans="1:11" ht="45" hidden="1" x14ac:dyDescent="0.25">
+    <row r="61" spans="1:14" ht="45" x14ac:dyDescent="0.25">
       <c r="A61" s="3" t="s">
         <v>95</v>
       </c>
@@ -3005,7 +3013,7 @@
         <v>46311</v>
       </c>
     </row>
-    <row r="62" spans="1:11" ht="60" hidden="1" x14ac:dyDescent="0.25">
+    <row r="62" spans="1:14" ht="60" x14ac:dyDescent="0.25">
       <c r="A62" s="3" t="s">
         <v>98</v>
       </c>
@@ -3038,7 +3046,7 @@
         <v>46311</v>
       </c>
     </row>
-    <row r="63" spans="1:11" ht="105" x14ac:dyDescent="0.25">
+    <row r="63" spans="1:14" ht="105" x14ac:dyDescent="0.25">
       <c r="A63" s="3" t="s">
         <v>89</v>
       </c>
@@ -3071,7 +3079,7 @@
         <v>46311</v>
       </c>
     </row>
-    <row r="64" spans="1:11" ht="105" hidden="1" x14ac:dyDescent="0.25">
+    <row r="64" spans="1:14" ht="105" x14ac:dyDescent="0.25">
       <c r="A64" s="3" t="s">
         <v>92</v>
       </c>
@@ -3137,7 +3145,7 @@
         <v>46311</v>
       </c>
     </row>
-    <row r="66" spans="1:11" ht="105" hidden="1" x14ac:dyDescent="0.25">
+    <row r="66" spans="1:11" ht="105" x14ac:dyDescent="0.25">
       <c r="A66" s="3" t="s">
         <v>98</v>
       </c>
@@ -3170,7 +3178,7 @@
         <v>46311</v>
       </c>
     </row>
-    <row r="67" spans="1:11" ht="75" hidden="1" x14ac:dyDescent="0.25">
+    <row r="67" spans="1:11" ht="75" x14ac:dyDescent="0.25">
       <c r="A67" s="3" t="s">
         <v>89</v>
       </c>
@@ -3203,7 +3211,7 @@
         <v>46311</v>
       </c>
     </row>
-    <row r="68" spans="1:11" ht="75" hidden="1" x14ac:dyDescent="0.25">
+    <row r="68" spans="1:11" ht="75" x14ac:dyDescent="0.25">
       <c r="A68" s="3" t="s">
         <v>92</v>
       </c>
@@ -3236,7 +3244,7 @@
         <v>46311</v>
       </c>
     </row>
-    <row r="69" spans="1:11" ht="120" hidden="1" x14ac:dyDescent="0.25">
+    <row r="69" spans="1:11" ht="120" x14ac:dyDescent="0.25">
       <c r="A69" s="3" t="s">
         <v>95</v>
       </c>
@@ -3269,7 +3277,7 @@
         <v>46311</v>
       </c>
     </row>
-    <row r="70" spans="1:11" ht="45" hidden="1" x14ac:dyDescent="0.25">
+    <row r="70" spans="1:11" ht="45" x14ac:dyDescent="0.25">
       <c r="A70" s="3" t="s">
         <v>95</v>
       </c>
@@ -3302,7 +3310,7 @@
         <v>46311</v>
       </c>
     </row>
-    <row r="71" spans="1:11" ht="60" hidden="1" x14ac:dyDescent="0.25">
+    <row r="71" spans="1:11" ht="60" x14ac:dyDescent="0.25">
       <c r="A71" s="3" t="s">
         <v>95</v>
       </c>
@@ -3335,7 +3343,7 @@
         <v>46311</v>
       </c>
     </row>
-    <row r="72" spans="1:11" ht="75" hidden="1" x14ac:dyDescent="0.25">
+    <row r="72" spans="1:11" ht="75" x14ac:dyDescent="0.25">
       <c r="A72" s="3" t="s">
         <v>95</v>
       </c>
@@ -3361,14 +3369,14 @@
         <v>120</v>
       </c>
       <c r="I72" s="5" t="s">
-        <v>157</v>
+        <v>156</v>
       </c>
       <c r="J72" s="3"/>
       <c r="K72" s="6">
         <v>46311</v>
       </c>
     </row>
-    <row r="73" spans="1:11" ht="75" hidden="1" x14ac:dyDescent="0.25">
+    <row r="73" spans="1:11" ht="75" x14ac:dyDescent="0.25">
       <c r="A73" s="3" t="s">
         <v>98</v>
       </c>
@@ -3401,7 +3409,7 @@
         <v>46311</v>
       </c>
     </row>
-    <row r="74" spans="1:11" ht="90" hidden="1" x14ac:dyDescent="0.25">
+    <row r="74" spans="1:11" ht="90" x14ac:dyDescent="0.25">
       <c r="A74" s="3" t="s">
         <v>89</v>
       </c>
@@ -3434,7 +3442,7 @@
         <v>46311</v>
       </c>
     </row>
-    <row r="75" spans="1:11" ht="90" hidden="1" x14ac:dyDescent="0.25">
+    <row r="75" spans="1:11" ht="90" x14ac:dyDescent="0.25">
       <c r="A75" s="3" t="s">
         <v>92</v>
       </c>
@@ -3467,7 +3475,7 @@
         <v>46311</v>
       </c>
     </row>
-    <row r="76" spans="1:11" ht="90" hidden="1" x14ac:dyDescent="0.25">
+    <row r="76" spans="1:11" ht="90" x14ac:dyDescent="0.25">
       <c r="A76" s="3" t="s">
         <v>95</v>
       </c>
@@ -3493,14 +3501,14 @@
         <v>120</v>
       </c>
       <c r="I76" s="5" t="s">
-        <v>157</v>
+        <v>156</v>
       </c>
       <c r="J76" s="3"/>
       <c r="K76" s="6">
         <v>46311</v>
       </c>
     </row>
-    <row r="77" spans="1:11" ht="90" hidden="1" x14ac:dyDescent="0.25">
+    <row r="77" spans="1:11" ht="90" x14ac:dyDescent="0.25">
       <c r="A77" s="3" t="s">
         <v>98</v>
       </c>
@@ -3533,7 +3541,7 @@
         <v>46311</v>
       </c>
     </row>
-    <row r="78" spans="1:11" ht="45" hidden="1" x14ac:dyDescent="0.25">
+    <row r="78" spans="1:11" ht="45" x14ac:dyDescent="0.25">
       <c r="A78" s="3" t="s">
         <v>98</v>
       </c>
@@ -3566,7 +3574,7 @@
         <v>46311</v>
       </c>
     </row>
-    <row r="79" spans="1:11" ht="90" hidden="1" x14ac:dyDescent="0.25">
+    <row r="79" spans="1:11" ht="90" x14ac:dyDescent="0.25">
       <c r="A79" s="3" t="s">
         <v>98</v>
       </c>
@@ -3599,7 +3607,7 @@
         <v>46311</v>
       </c>
     </row>
-    <row r="80" spans="1:11" ht="45" hidden="1" x14ac:dyDescent="0.25">
+    <row r="80" spans="1:11" ht="45" x14ac:dyDescent="0.25">
       <c r="A80" s="3" t="s">
         <v>98</v>
       </c>
@@ -3632,7 +3640,7 @@
         <v>46311</v>
       </c>
     </row>
-    <row r="81" spans="1:11" ht="90" hidden="1" x14ac:dyDescent="0.25">
+    <row r="81" spans="1:11" ht="90" x14ac:dyDescent="0.25">
       <c r="A81" s="3" t="s">
         <v>89</v>
       </c>
@@ -3665,7 +3673,7 @@
         <v>46311</v>
       </c>
     </row>
-    <row r="82" spans="1:11" ht="90" hidden="1" x14ac:dyDescent="0.25">
+    <row r="82" spans="1:11" ht="90" x14ac:dyDescent="0.25">
       <c r="A82" s="3" t="s">
         <v>92</v>
       </c>
@@ -3698,7 +3706,7 @@
         <v>46311</v>
       </c>
     </row>
-    <row r="83" spans="1:11" ht="90" hidden="1" x14ac:dyDescent="0.25">
+    <row r="83" spans="1:11" ht="90" x14ac:dyDescent="0.25">
       <c r="A83" s="3" t="s">
         <v>95</v>
       </c>
@@ -3724,14 +3732,14 @@
         <v>120</v>
       </c>
       <c r="I83" s="5" t="s">
-        <v>157</v>
+        <v>156</v>
       </c>
       <c r="J83" s="3"/>
       <c r="K83" s="6">
         <v>46311</v>
       </c>
     </row>
-    <row r="84" spans="1:11" ht="90" hidden="1" x14ac:dyDescent="0.25">
+    <row r="84" spans="1:11" ht="90" x14ac:dyDescent="0.25">
       <c r="A84" s="3" t="s">
         <v>98</v>
       </c>
@@ -3764,7 +3772,7 @@
         <v>46311</v>
       </c>
     </row>
-    <row r="85" spans="1:11" ht="75" hidden="1" x14ac:dyDescent="0.25">
+    <row r="85" spans="1:11" ht="75" x14ac:dyDescent="0.25">
       <c r="A85" s="3" t="s">
         <v>89</v>
       </c>
@@ -3797,7 +3805,7 @@
         <v>46311</v>
       </c>
     </row>
-    <row r="86" spans="1:11" ht="75" hidden="1" x14ac:dyDescent="0.25">
+    <row r="86" spans="1:11" ht="75" x14ac:dyDescent="0.25">
       <c r="A86" s="3" t="s">
         <v>92</v>
       </c>
@@ -3830,7 +3838,7 @@
         <v>46311</v>
       </c>
     </row>
-    <row r="87" spans="1:11" ht="60" hidden="1" x14ac:dyDescent="0.25">
+    <row r="87" spans="1:11" ht="60" x14ac:dyDescent="0.25">
       <c r="A87" s="3" t="s">
         <v>98</v>
       </c>
@@ -3863,7 +3871,7 @@
         <v>46311</v>
       </c>
     </row>
-    <row r="88" spans="1:11" ht="120" hidden="1" x14ac:dyDescent="0.25">
+    <row r="88" spans="1:11" ht="120" x14ac:dyDescent="0.25">
       <c r="A88" s="3" t="s">
         <v>98</v>
       </c>
@@ -3896,7 +3904,7 @@
         <v>46311</v>
       </c>
     </row>
-    <row r="89" spans="1:11" ht="45" hidden="1" x14ac:dyDescent="0.25">
+    <row r="89" spans="1:11" ht="45" x14ac:dyDescent="0.25">
       <c r="A89" s="3" t="s">
         <v>98</v>
       </c>
@@ -3929,7 +3937,7 @@
         <v>46311</v>
       </c>
     </row>
-    <row r="90" spans="1:11" ht="60" hidden="1" x14ac:dyDescent="0.25">
+    <row r="90" spans="1:11" ht="60" x14ac:dyDescent="0.25">
       <c r="A90" s="3" t="s">
         <v>98</v>
       </c>
@@ -3962,7 +3970,7 @@
         <v>46311</v>
       </c>
     </row>
-    <row r="91" spans="1:11" ht="75" hidden="1" x14ac:dyDescent="0.25">
+    <row r="91" spans="1:11" ht="75" x14ac:dyDescent="0.25">
       <c r="A91" s="3" t="s">
         <v>95</v>
       </c>
@@ -3988,14 +3996,14 @@
         <v>120</v>
       </c>
       <c r="I91" s="5" t="s">
-        <v>157</v>
+        <v>156</v>
       </c>
       <c r="J91" s="3"/>
       <c r="K91" s="6">
         <v>46311</v>
       </c>
     </row>
-    <row r="92" spans="1:11" ht="75" hidden="1" x14ac:dyDescent="0.25">
+    <row r="92" spans="1:11" ht="75" x14ac:dyDescent="0.25">
       <c r="A92" s="3" t="s">
         <v>98</v>
       </c>
@@ -4028,7 +4036,7 @@
         <v>46311</v>
       </c>
     </row>
-    <row r="93" spans="1:11" ht="90" hidden="1" x14ac:dyDescent="0.25">
+    <row r="93" spans="1:11" ht="90" x14ac:dyDescent="0.25">
       <c r="A93" s="3" t="s">
         <v>89</v>
       </c>
@@ -4061,7 +4069,7 @@
         <v>46311</v>
       </c>
     </row>
-    <row r="94" spans="1:11" ht="90" hidden="1" x14ac:dyDescent="0.25">
+    <row r="94" spans="1:11" ht="90" x14ac:dyDescent="0.25">
       <c r="A94" s="3" t="s">
         <v>92</v>
       </c>
@@ -4094,7 +4102,7 @@
         <v>46311</v>
       </c>
     </row>
-    <row r="95" spans="1:11" ht="90" hidden="1" x14ac:dyDescent="0.25">
+    <row r="95" spans="1:11" ht="90" x14ac:dyDescent="0.25">
       <c r="A95" s="3" t="s">
         <v>95</v>
       </c>
@@ -4120,14 +4128,14 @@
         <v>123</v>
       </c>
       <c r="I95" s="5" t="s">
-        <v>158</v>
+        <v>157</v>
       </c>
       <c r="J95" s="3"/>
       <c r="K95" s="6">
         <v>46311</v>
       </c>
     </row>
-    <row r="96" spans="1:11" ht="90" hidden="1" x14ac:dyDescent="0.25">
+    <row r="96" spans="1:11" ht="90" x14ac:dyDescent="0.25">
       <c r="A96" s="3" t="s">
         <v>98</v>
       </c>
@@ -4161,11 +4169,7 @@
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:K96" xr:uid="{00000000-0009-0000-0000-000000000000}">
-    <filterColumn colId="8">
-      <filters blank="1"/>
-    </filterColumn>
-  </autoFilter>
+  <autoFilter ref="A1:K96" xr:uid="{00000000-0009-0000-0000-000000000000}"/>
   <dataValidations count="1">
     <dataValidation type="list" allowBlank="1" error="Escolha um status da lista." sqref="H2:H37 H39:H96" xr:uid="{00000000-0002-0000-0000-000000000000}">
       <formula1>"ATENDE,ATENDE_PARCIALMENTE,NAO_ATENDE,NAO_SEI"</formula1>
@@ -4213,55 +4217,57 @@
     <hyperlink ref="I69" r:id="rId39" display="https://transparencianovo.ib.itaborai.rj.gov.br/ouvidoria/" xr:uid="{2A07D261-D84E-4400-8D9D-9C1C2D28594B}"/>
     <hyperlink ref="I88" r:id="rId40" display="https://transparencianovo.ib.itaborai.rj.gov.br/ouvidoria/" xr:uid="{AFBEB50C-B1AA-44EF-B1F2-8159A7DC4E58}"/>
     <hyperlink ref="I32" r:id="rId41" display="https://portal.duquedecaxias.rj.gov.br/" xr:uid="{70142200-4705-4AE1-A7E7-65C2090D4D05}"/>
-    <hyperlink ref="I51" r:id="rId42" display="https://japeri.rj.gov.br/" xr:uid="{343DE6A2-18DB-45E8-9C22-68AE9F3C4BF8}"/>
-    <hyperlink ref="I70" r:id="rId43" display="https://site.ib.itaborai.rj.gov.br/" xr:uid="{2D6848F4-C6D0-4D4A-AAE5-FEBA31C1C9FB}"/>
-    <hyperlink ref="I89" r:id="rId44" display="https://site.ib.itaborai.rj.gov.br/" xr:uid="{14544C5E-8DB6-40C7-B9F9-9000B3ABDBC8}"/>
-    <hyperlink ref="I71" r:id="rId45" display="https://site.ib.itaborai.rj.gov.br/" xr:uid="{229306A2-FA9F-42AA-B7CC-F26ECDC1145C}"/>
-    <hyperlink ref="I33" r:id="rId46" display="https://portal.duquedecaxias.rj.gov.br/" xr:uid="{69A15AC1-D494-4D4A-B45F-7AD990691CA9}"/>
-    <hyperlink ref="I29" r:id="rId47" display="https://transparencia.duquedecaxias.rj.gov.br/" xr:uid="{9DE67E03-8D6A-4064-A132-C2356FF0DC80}"/>
-    <hyperlink ref="I34" r:id="rId48" display="https://japeri.rj.gov.br/service/lgpd/" xr:uid="{2C2F72F6-B686-40F4-B210-D55C31E3C177}"/>
-    <hyperlink ref="I36" r:id="rId49" location="/VZIcwd3tEQSz63QIK2HkQw==*/lgpd" display="https://transparencia.betha.cloud/ - /VZIcwd3tEQSz63QIK2HkQw==*/lgpd" xr:uid="{1B1BB63C-94CA-4D89-8861-C0D8C7806BD8}"/>
-    <hyperlink ref="I35" r:id="rId50" display="https://transparencianovo.ib.itaborai.rj.gov.br/lgpd-encarregado-de-dados/" xr:uid="{B2BE9470-D315-4276-A126-877B8241DA24}"/>
-    <hyperlink ref="I67" r:id="rId51" display="https://transparencia.duquedecaxias.rj.gov.br/" xr:uid="{06D0CF86-93A3-45CF-9EEB-46354341C5F1}"/>
-    <hyperlink ref="I68" r:id="rId52" display="https://japeri.geosiap.net.br/portal-transparencia/execucao/despesas-detalhadas" xr:uid="{526DB44C-0D3F-4CDA-ADA8-4B256E9BBBF2}"/>
-    <hyperlink ref="I73" r:id="rId53" location="/VZIcwd3tEQSz63QIK2HkQw==*/consulta/31210" display="https://transparencia.betha.cloud/ - /VZIcwd3tEQSz63QIK2HkQw==*/consulta/31210" xr:uid="{7FCCC53A-F492-4CFF-8F37-A2A4D7251887}"/>
-    <hyperlink ref="I72" r:id="rId54" display="https://itaborai.supernova.com.br:8443/contaspublicas/despesa.xhtml?exercicio=2026" xr:uid="{491D35D6-9B6B-4B98-8F45-2C9DF4414230}"/>
-    <hyperlink ref="I76" r:id="rId55" display="https://itaborai.supernova.com.br:8443/contaspublicas/despesa.xhtml?exercicio=2026" xr:uid="{FED8B7F6-3A0B-44E2-BE39-350434C7785D}"/>
-    <hyperlink ref="I77" r:id="rId56" location="/VZIcwd3tEQSz63QIK2HkQw==*/consulta/31210" display="https://transparencia.betha.cloud/ - /VZIcwd3tEQSz63QIK2HkQw==*/consulta/31210" xr:uid="{0952FC34-C48C-480C-9B05-EB221EE5974D}"/>
-    <hyperlink ref="I75" r:id="rId57" display="https://japeri.geosiap.net.br/portal-transparencia/execucao/despesas-detalhadas" xr:uid="{FB220F20-2671-40B6-A481-144D82302FB0}"/>
-    <hyperlink ref="I74" r:id="rId58" display="https://transparencia.duquedecaxias.rj.gov.br/" xr:uid="{C0B8A588-C63C-43EA-BBDE-644B28BB0CBE}"/>
-    <hyperlink ref="I84" r:id="rId59" location="/VZIcwd3tEQSz63QIK2HkQw==*/consulta/31210" display="https://transparencia.betha.cloud/ - /VZIcwd3tEQSz63QIK2HkQw==*/consulta/31210" xr:uid="{0D2B01D7-89B0-4CFA-933C-0D4B6A1ACCFD}"/>
-    <hyperlink ref="I83" r:id="rId60" display="https://itaborai.supernova.com.br:8443/contaspublicas/despesa.xhtml?exercicio=2026" xr:uid="{8A48F905-741C-418E-BA5E-4693660D3D33}"/>
-    <hyperlink ref="I82" r:id="rId61" display="https://japeri.geosiap.net.br/portal-transparencia/execucao/despesas-detalhadas" xr:uid="{ABDF5C98-E226-4093-B342-30C3D8C6A0BD}"/>
-    <hyperlink ref="I81" r:id="rId62" display="https://transparencia.duquedecaxias.rj.gov.br/" xr:uid="{8FDD6BCA-61ED-4310-AEF5-BF641D16D97E}"/>
-    <hyperlink ref="I85" r:id="rId63" display="https://transparencia.duquedecaxias.rj.gov.br/" xr:uid="{3F5AD71F-1627-407F-B4A7-07905337B029}"/>
-    <hyperlink ref="I91" r:id="rId64" display="https://itaborai.supernova.com.br:8443/contaspublicas/relacao_funcionarios.xhtml?exercicio=2026" xr:uid="{FD3B830E-2850-41C6-A557-36A65720152D}"/>
-    <hyperlink ref="I86" r:id="rId65" display="https://japeri.geosiap.net.br/portal-transparencia/rh/servidores/ativos" xr:uid="{9A8A60B4-86F6-4496-AE68-CCC9DC47094C}"/>
-    <hyperlink ref="I92" r:id="rId66" location="/VZIcwd3tEQSz63QIK2HkQw==*/consulta/406074" display="https://transparencia.betha.cloud/ - /VZIcwd3tEQSz63QIK2HkQw==*/consulta/406074" xr:uid="{8723CA43-BB98-4C9C-8E47-00F11A32E4B7}"/>
-    <hyperlink ref="I96" r:id="rId67" location="/VZIcwd3tEQSz63QIK2HkQw==*/consulta/31197" display="https://transparencia.betha.cloud/ - /VZIcwd3tEQSz63QIK2HkQw==*/consulta/31197" xr:uid="{8655B222-5D9A-4E66-84A2-13E003E492F8}"/>
-    <hyperlink ref="I95" r:id="rId68" display="https://transparencianovo.ib.itaborai.rj.gov.br/editais-e-atos-juridicos/licitacoes/" xr:uid="{599716B6-A63F-483E-86CE-8D91FB2B281A}"/>
-    <hyperlink ref="I94" r:id="rId69" display="https://japeri.geosiap.net.br/portal-transparencia/licitacoes/licitacoes" xr:uid="{7D72FB8D-643B-43AB-958C-DA7EEC919E85}"/>
-    <hyperlink ref="I93" r:id="rId70" display="https://transparencia.duquedecaxias.rj.gov.br/" xr:uid="{83B05EE5-F6E9-4E03-B196-C3D882C358AF}"/>
-    <hyperlink ref="I37" r:id="rId71" display="https://transparencia.duquedecaxias.rj.gov.br/" xr:uid="{FEC15298-1DC5-4075-B2E3-D3F1D406F342}"/>
-    <hyperlink ref="I38" r:id="rId72" display="https://japeri.geosiap.net.br/portal-transparencia/publicacoes?id_publicacao_tipo=7" xr:uid="{2B442C9F-C75E-4A97-84A2-5FA81EF1B030}"/>
-    <hyperlink ref="I43" r:id="rId73" location="/VZIcwd3tEQSz63QIK2HkQw==*/dados-abertos" display="https://transparencia.betha.cloud/ - /VZIcwd3tEQSz63QIK2HkQw==*/dados-abertos" xr:uid="{2413ACF4-05D9-4480-8988-5BAA5D63F15B}"/>
-    <hyperlink ref="I44" r:id="rId74" display="https://transparencia.duquedecaxias.rj.gov.br/" xr:uid="{F3EDE991-0D9F-46F7-9BE5-407292D0DB42}"/>
-    <hyperlink ref="I45" r:id="rId75" display="https://japeri.geosiap.net.br/portal-transparencia/publicacoes?id_publicacao_sub_tipo=5" xr:uid="{AF467312-E4EA-4641-94D8-C2304E41D9A3}"/>
-    <hyperlink ref="I46" r:id="rId76" display="https://transparencianovo.ib.itaborai.rj.gov.br/instrumentos-de-planejamento-da-gestao/loa/" xr:uid="{5D335BD9-6678-4AF4-B848-485C063D11D0}"/>
-    <hyperlink ref="I47" r:id="rId77" location="/VZIcwd3tEQSz63QIK2HkQw==*/consulta/191443" display="https://transparencia.betha.cloud/ - /VZIcwd3tEQSz63QIK2HkQw==*/consulta/191443" xr:uid="{C4720769-FB8E-4E41-8E82-972F0403E190}"/>
-    <hyperlink ref="I57" r:id="rId78" display="https://japeri.geosiap.net.br/portal-transparencia/publicacoes?id_publicacao_sub_tipo=4" xr:uid="{E64D6C6B-4B1E-41FA-B166-03E1F7856650}"/>
-    <hyperlink ref="I62" r:id="rId79" location="/VZIcwd3tEQSz63QIK2HkQw==*/consulta/195138" display="https://transparencia.betha.cloud/ - /VZIcwd3tEQSz63QIK2HkQw==*/consulta/195138" xr:uid="{A11B6567-65E1-4A80-8622-0A6C7EF1871F}"/>
-    <hyperlink ref="I58" r:id="rId80" display="https://transparencianovo.ib.itaborai.rj.gov.br/15-relatorios-fiscais-da-lrf/rreo/" xr:uid="{86255E59-7D44-4BA0-AB8F-218DB1F43FBE}"/>
-    <hyperlink ref="I56" r:id="rId81" display="https://transparencia.duquedecaxias.rj.gov.br/" xr:uid="{FA59F9C4-AC02-4B0B-9B89-431DA1FF6AC9}"/>
-    <hyperlink ref="I66" r:id="rId82" location="/VZIcwd3tEQSz63QIK2HkQw==*/consulta/195138" display="https://transparencia.betha.cloud/ - /VZIcwd3tEQSz63QIK2HkQw==*/consulta/195138" xr:uid="{A0E415DB-AACC-41CC-B4B8-7756CC02B1FA}"/>
-    <hyperlink ref="I64" r:id="rId83" display="https://japeri.geosiap.net.br/portal-transparencia/publicacoes?id_publicacao_sub_tipo=4" xr:uid="{B32052E9-2098-488E-BD9B-0C8A77CBE414}"/>
-    <hyperlink ref="F53" r:id="rId84" xr:uid="{F8A7FA24-762B-4564-B5F3-8978CDD38E9C}"/>
-    <hyperlink ref="I54" r:id="rId85" display="https://site.ib.itaborai.rj.gov.br/" xr:uid="{8B499DD7-5B58-4072-929E-425F41FB48D5}"/>
-    <hyperlink ref="I53" r:id="rId86" display="https://japeri.rj.gov.br/contato/" xr:uid="{EA0DB2E7-AA2A-4E14-A0F4-CA1612C1BF96}"/>
-    <hyperlink ref="I55" r:id="rId87" display="https://falabr.cgu.gov.br/v2/" xr:uid="{AAF18F11-8D25-4476-920D-42DA5D55562E}"/>
-    <hyperlink ref="I48" r:id="rId88" display="https://transparencia.duquedecaxias.rj.gov.br/?serv=1473" xr:uid="{93F38728-2763-4CF0-88C7-1EF465BF0B96}"/>
-    <hyperlink ref="I9" r:id="rId89" display="https://transparencia.prefeitura.rio/servidor-municipal/" xr:uid="{F3C8FF16-043F-4D3E-ADC7-989E4A4F4866}"/>
-    <hyperlink ref="I39" r:id="rId90" display="https://transparencianovo.ib.itaborai.rj.gov.br/" xr:uid="{817723A9-3570-487A-9170-3453AD1D7CF2}"/>
+    <hyperlink ref="I70" r:id="rId42" display="https://site.ib.itaborai.rj.gov.br/" xr:uid="{2D6848F4-C6D0-4D4A-AAE5-FEBA31C1C9FB}"/>
+    <hyperlink ref="I89" r:id="rId43" display="https://site.ib.itaborai.rj.gov.br/" xr:uid="{14544C5E-8DB6-40C7-B9F9-9000B3ABDBC8}"/>
+    <hyperlink ref="I71" r:id="rId44" display="https://site.ib.itaborai.rj.gov.br/" xr:uid="{229306A2-FA9F-42AA-B7CC-F26ECDC1145C}"/>
+    <hyperlink ref="I33" r:id="rId45" display="https://portal.duquedecaxias.rj.gov.br/" xr:uid="{69A15AC1-D494-4D4A-B45F-7AD990691CA9}"/>
+    <hyperlink ref="I29" r:id="rId46" display="https://transparencia.duquedecaxias.rj.gov.br/" xr:uid="{9DE67E03-8D6A-4064-A132-C2356FF0DC80}"/>
+    <hyperlink ref="I34" r:id="rId47" display="https://japeri.rj.gov.br/service/lgpd/" xr:uid="{2C2F72F6-B686-40F4-B210-D55C31E3C177}"/>
+    <hyperlink ref="I36" r:id="rId48" location="/VZIcwd3tEQSz63QIK2HkQw==*/lgpd" display="https://transparencia.betha.cloud/ - /VZIcwd3tEQSz63QIK2HkQw==*/lgpd" xr:uid="{1B1BB63C-94CA-4D89-8861-C0D8C7806BD8}"/>
+    <hyperlink ref="I35" r:id="rId49" display="https://transparencianovo.ib.itaborai.rj.gov.br/lgpd-encarregado-de-dados/" xr:uid="{B2BE9470-D315-4276-A126-877B8241DA24}"/>
+    <hyperlink ref="I67" r:id="rId50" display="https://transparencia.duquedecaxias.rj.gov.br/" xr:uid="{06D0CF86-93A3-45CF-9EEB-46354341C5F1}"/>
+    <hyperlink ref="I68" r:id="rId51" display="https://japeri.geosiap.net.br/portal-transparencia/execucao/despesas-detalhadas" xr:uid="{526DB44C-0D3F-4CDA-ADA8-4B256E9BBBF2}"/>
+    <hyperlink ref="I73" r:id="rId52" location="/VZIcwd3tEQSz63QIK2HkQw==*/consulta/31210" display="https://transparencia.betha.cloud/ - /VZIcwd3tEQSz63QIK2HkQw==*/consulta/31210" xr:uid="{7FCCC53A-F492-4CFF-8F37-A2A4D7251887}"/>
+    <hyperlink ref="I72" r:id="rId53" display="https://itaborai.supernova.com.br:8443/contaspublicas/despesa.xhtml?exercicio=2026" xr:uid="{491D35D6-9B6B-4B98-8F45-2C9DF4414230}"/>
+    <hyperlink ref="I76" r:id="rId54" display="https://itaborai.supernova.com.br:8443/contaspublicas/despesa.xhtml?exercicio=2026" xr:uid="{FED8B7F6-3A0B-44E2-BE39-350434C7785D}"/>
+    <hyperlink ref="I77" r:id="rId55" location="/VZIcwd3tEQSz63QIK2HkQw==*/consulta/31210" display="https://transparencia.betha.cloud/ - /VZIcwd3tEQSz63QIK2HkQw==*/consulta/31210" xr:uid="{0952FC34-C48C-480C-9B05-EB221EE5974D}"/>
+    <hyperlink ref="I75" r:id="rId56" display="https://japeri.geosiap.net.br/portal-transparencia/execucao/despesas-detalhadas" xr:uid="{FB220F20-2671-40B6-A481-144D82302FB0}"/>
+    <hyperlink ref="I74" r:id="rId57" display="https://transparencia.duquedecaxias.rj.gov.br/" xr:uid="{C0B8A588-C63C-43EA-BBDE-644B28BB0CBE}"/>
+    <hyperlink ref="I84" r:id="rId58" location="/VZIcwd3tEQSz63QIK2HkQw==*/consulta/31210" display="https://transparencia.betha.cloud/ - /VZIcwd3tEQSz63QIK2HkQw==*/consulta/31210" xr:uid="{0D2B01D7-89B0-4CFA-933C-0D4B6A1ACCFD}"/>
+    <hyperlink ref="I83" r:id="rId59" display="https://itaborai.supernova.com.br:8443/contaspublicas/despesa.xhtml?exercicio=2026" xr:uid="{8A48F905-741C-418E-BA5E-4693660D3D33}"/>
+    <hyperlink ref="I82" r:id="rId60" display="https://japeri.geosiap.net.br/portal-transparencia/execucao/despesas-detalhadas" xr:uid="{ABDF5C98-E226-4093-B342-30C3D8C6A0BD}"/>
+    <hyperlink ref="I81" r:id="rId61" display="https://transparencia.duquedecaxias.rj.gov.br/" xr:uid="{8FDD6BCA-61ED-4310-AEF5-BF641D16D97E}"/>
+    <hyperlink ref="I85" r:id="rId62" display="https://transparencia.duquedecaxias.rj.gov.br/" xr:uid="{3F5AD71F-1627-407F-B4A7-07905337B029}"/>
+    <hyperlink ref="I91" r:id="rId63" display="https://itaborai.supernova.com.br:8443/contaspublicas/relacao_funcionarios.xhtml?exercicio=2026" xr:uid="{FD3B830E-2850-41C6-A557-36A65720152D}"/>
+    <hyperlink ref="I86" r:id="rId64" display="https://japeri.geosiap.net.br/portal-transparencia/rh/servidores/ativos" xr:uid="{9A8A60B4-86F6-4496-AE68-CCC9DC47094C}"/>
+    <hyperlink ref="I92" r:id="rId65" location="/VZIcwd3tEQSz63QIK2HkQw==*/consulta/406074" display="https://transparencia.betha.cloud/ - /VZIcwd3tEQSz63QIK2HkQw==*/consulta/406074" xr:uid="{8723CA43-BB98-4C9C-8E47-00F11A32E4B7}"/>
+    <hyperlink ref="I96" r:id="rId66" location="/VZIcwd3tEQSz63QIK2HkQw==*/consulta/31197" display="https://transparencia.betha.cloud/ - /VZIcwd3tEQSz63QIK2HkQw==*/consulta/31197" xr:uid="{8655B222-5D9A-4E66-84A2-13E003E492F8}"/>
+    <hyperlink ref="I95" r:id="rId67" display="https://transparencianovo.ib.itaborai.rj.gov.br/editais-e-atos-juridicos/licitacoes/" xr:uid="{599716B6-A63F-483E-86CE-8D91FB2B281A}"/>
+    <hyperlink ref="I94" r:id="rId68" display="https://japeri.geosiap.net.br/portal-transparencia/licitacoes/licitacoes" xr:uid="{7D72FB8D-643B-43AB-958C-DA7EEC919E85}"/>
+    <hyperlink ref="I93" r:id="rId69" display="https://transparencia.duquedecaxias.rj.gov.br/" xr:uid="{83B05EE5-F6E9-4E03-B196-C3D882C358AF}"/>
+    <hyperlink ref="I37" r:id="rId70" display="https://transparencia.duquedecaxias.rj.gov.br/" xr:uid="{FEC15298-1DC5-4075-B2E3-D3F1D406F342}"/>
+    <hyperlink ref="I38" r:id="rId71" display="https://japeri.geosiap.net.br/portal-transparencia/publicacoes?id_publicacao_tipo=7" xr:uid="{2B442C9F-C75E-4A97-84A2-5FA81EF1B030}"/>
+    <hyperlink ref="I43" r:id="rId72" location="/VZIcwd3tEQSz63QIK2HkQw==*/dados-abertos" display="https://transparencia.betha.cloud/ - /VZIcwd3tEQSz63QIK2HkQw==*/dados-abertos" xr:uid="{2413ACF4-05D9-4480-8988-5BAA5D63F15B}"/>
+    <hyperlink ref="I44" r:id="rId73" display="https://transparencia.duquedecaxias.rj.gov.br/" xr:uid="{F3EDE991-0D9F-46F7-9BE5-407292D0DB42}"/>
+    <hyperlink ref="I45" r:id="rId74" display="https://japeri.geosiap.net.br/portal-transparencia/publicacoes?id_publicacao_sub_tipo=5" xr:uid="{AF467312-E4EA-4641-94D8-C2304E41D9A3}"/>
+    <hyperlink ref="I46" r:id="rId75" display="https://transparencianovo.ib.itaborai.rj.gov.br/instrumentos-de-planejamento-da-gestao/loa/" xr:uid="{5D335BD9-6678-4AF4-B848-485C063D11D0}"/>
+    <hyperlink ref="I47" r:id="rId76" location="/VZIcwd3tEQSz63QIK2HkQw==*/consulta/191443" display="https://transparencia.betha.cloud/ - /VZIcwd3tEQSz63QIK2HkQw==*/consulta/191443" xr:uid="{C4720769-FB8E-4E41-8E82-972F0403E190}"/>
+    <hyperlink ref="I57" r:id="rId77" display="https://japeri.geosiap.net.br/portal-transparencia/publicacoes?id_publicacao_sub_tipo=4" xr:uid="{E64D6C6B-4B1E-41FA-B166-03E1F7856650}"/>
+    <hyperlink ref="I62" r:id="rId78" location="/VZIcwd3tEQSz63QIK2HkQw==*/consulta/195138" display="https://transparencia.betha.cloud/ - /VZIcwd3tEQSz63QIK2HkQw==*/consulta/195138" xr:uid="{A11B6567-65E1-4A80-8622-0A6C7EF1871F}"/>
+    <hyperlink ref="I58" r:id="rId79" display="https://transparencianovo.ib.itaborai.rj.gov.br/15-relatorios-fiscais-da-lrf/rreo/" xr:uid="{86255E59-7D44-4BA0-AB8F-218DB1F43FBE}"/>
+    <hyperlink ref="I56" r:id="rId80" display="https://transparencia.duquedecaxias.rj.gov.br/" xr:uid="{FA59F9C4-AC02-4B0B-9B89-431DA1FF6AC9}"/>
+    <hyperlink ref="I66" r:id="rId81" location="/VZIcwd3tEQSz63QIK2HkQw==*/consulta/195138" display="https://transparencia.betha.cloud/ - /VZIcwd3tEQSz63QIK2HkQw==*/consulta/195138" xr:uid="{A0E415DB-AACC-41CC-B4B8-7756CC02B1FA}"/>
+    <hyperlink ref="I64" r:id="rId82" display="https://japeri.geosiap.net.br/portal-transparencia/publicacoes?id_publicacao_sub_tipo=4" xr:uid="{B32052E9-2098-488E-BD9B-0C8A77CBE414}"/>
+    <hyperlink ref="F53" r:id="rId83" xr:uid="{F8A7FA24-762B-4564-B5F3-8978CDD38E9C}"/>
+    <hyperlink ref="I54" r:id="rId84" display="https://site.ib.itaborai.rj.gov.br/" xr:uid="{8B499DD7-5B58-4072-929E-425F41FB48D5}"/>
+    <hyperlink ref="I53" r:id="rId85" display="https://japeri.rj.gov.br/contato/" xr:uid="{EA0DB2E7-AA2A-4E14-A0F4-CA1612C1BF96}"/>
+    <hyperlink ref="I55" r:id="rId86" display="https://falabr.cgu.gov.br/v2/" xr:uid="{AAF18F11-8D25-4476-920D-42DA5D55562E}"/>
+    <hyperlink ref="I48" r:id="rId87" display="https://transparencia.duquedecaxias.rj.gov.br/?serv=1473" xr:uid="{93F38728-2763-4CF0-88C7-1EF465BF0B96}"/>
+    <hyperlink ref="I9" r:id="rId88" display="https://transparencia.prefeitura.rio/servidor-municipal/" xr:uid="{F3C8FF16-043F-4D3E-ADC7-989E4A4F4866}"/>
+    <hyperlink ref="I39" r:id="rId89" display="https://transparencianovo.ib.itaborai.rj.gov.br/" xr:uid="{817723A9-3570-487A-9170-3453AD1D7CF2}"/>
+    <hyperlink ref="I50" r:id="rId90" display="https://falabr.cgu.gov.br/v2/?uf=rj&amp;municipio=japeri" xr:uid="{2DC6F6BD-0423-434D-A4AB-97C0D2F52179}"/>
+    <hyperlink ref="I51" r:id="rId91" display="https://japeri.geosiap.net.br/portal-transparencia/home" xr:uid="{B88C8163-68DC-4DAF-81B7-496ACEC4E2D0}"/>
+    <hyperlink ref="I52" r:id="rId92" display="https://japeri.geosiap.net.br/portal-transparencia/home" xr:uid="{DDDB96B2-5EB2-49CB-9AFA-DF53EE4726B3}"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
test(golden): revisa rótulo 1.2 do Rio (ícone de transparência no topo)
</commit_message>
<xml_diff>
--- a/golden/golden_set.xlsx
+++ b/golden/golden_set.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Gerson\Documents\CASE MPRJ 2026\monitor-transparencia\golden\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9E4145CC-3ACB-4671-9104-774211C210F0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5C23757A-BAC5-41A4-8607-E064C50B7810}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="14400" yWindow="0" windowWidth="14400" windowHeight="15600" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="rotulos" sheetId="1" r:id="rId1"/>
@@ -430,9 +430,6 @@
     <t>ATENDE_PARCIALMENTE</t>
   </si>
   <si>
-    <t>o link está no rodapé da página</t>
-  </si>
-  <si>
     <t>ferramenta de busca no topo da página</t>
   </si>
   <si>
@@ -557,6 +554,9 @@
   </si>
   <si>
     <t>revisada em 16/10/2026: identificado texto no topo da página</t>
+  </si>
+  <si>
+    <t>revisada em 16/10/2026: há icone no inicio da página</t>
   </si>
 </sst>
 </file>
@@ -1064,13 +1064,13 @@
         <v>17</v>
       </c>
       <c r="H3" s="3" t="s">
-        <v>123</v>
+        <v>120</v>
       </c>
       <c r="I3" s="5" t="s">
         <v>121</v>
       </c>
       <c r="J3" s="3" t="s">
-        <v>124</v>
+        <v>166</v>
       </c>
       <c r="K3" s="6">
         <v>46309</v>
@@ -1105,7 +1105,7 @@
         <v>121</v>
       </c>
       <c r="J4" s="3" t="s">
-        <v>125</v>
+        <v>124</v>
       </c>
       <c r="K4" s="6">
         <v>46309</v>
@@ -1140,7 +1140,7 @@
         <v>121</v>
       </c>
       <c r="J5" s="3" t="s">
-        <v>126</v>
+        <v>125</v>
       </c>
       <c r="K5" s="6">
         <v>46309</v>
@@ -1172,10 +1172,10 @@
         <v>120</v>
       </c>
       <c r="I6" s="5" t="s">
-        <v>128</v>
+        <v>127</v>
       </c>
       <c r="J6" s="3" t="s">
-        <v>127</v>
+        <v>126</v>
       </c>
       <c r="K6" s="6">
         <v>46309</v>
@@ -1207,7 +1207,7 @@
         <v>120</v>
       </c>
       <c r="I7" s="5" t="s">
-        <v>128</v>
+        <v>127</v>
       </c>
       <c r="J7" s="3"/>
       <c r="K7" s="6">
@@ -1240,10 +1240,10 @@
         <v>120</v>
       </c>
       <c r="I8" s="5" t="s">
+        <v>127</v>
+      </c>
+      <c r="J8" s="3" t="s">
         <v>128</v>
-      </c>
-      <c r="J8" s="3" t="s">
-        <v>129</v>
       </c>
       <c r="K8" s="7">
         <v>46309</v>
@@ -1272,13 +1272,13 @@
         <v>17</v>
       </c>
       <c r="H9" s="3" t="s">
+        <v>129</v>
+      </c>
+      <c r="I9" s="5" t="s">
+        <v>163</v>
+      </c>
+      <c r="J9" s="3" t="s">
         <v>130</v>
-      </c>
-      <c r="I9" s="5" t="s">
-        <v>164</v>
-      </c>
-      <c r="J9" s="3" t="s">
-        <v>131</v>
       </c>
       <c r="K9" s="8">
         <v>46309</v>
@@ -1307,13 +1307,13 @@
         <v>17</v>
       </c>
       <c r="H10" s="3" t="s">
-        <v>130</v>
+        <v>129</v>
       </c>
       <c r="I10" s="5" t="s">
+        <v>131</v>
+      </c>
+      <c r="J10" s="3" t="s">
         <v>132</v>
-      </c>
-      <c r="J10" s="3" t="s">
-        <v>133</v>
       </c>
       <c r="K10" s="8">
         <v>46309</v>
@@ -1345,10 +1345,10 @@
         <v>120</v>
       </c>
       <c r="I11" s="5" t="s">
+        <v>133</v>
+      </c>
+      <c r="J11" s="3" t="s">
         <v>134</v>
-      </c>
-      <c r="J11" s="3" t="s">
-        <v>135</v>
       </c>
       <c r="K11" s="8">
         <v>46309</v>
@@ -1377,13 +1377,13 @@
         <v>17</v>
       </c>
       <c r="H12" s="3" t="s">
-        <v>130</v>
+        <v>129</v>
       </c>
       <c r="I12" s="5" t="s">
+        <v>135</v>
+      </c>
+      <c r="J12" s="3" t="s">
         <v>136</v>
-      </c>
-      <c r="J12" s="3" t="s">
-        <v>137</v>
       </c>
       <c r="K12" s="8">
         <v>46309</v>
@@ -1514,7 +1514,7 @@
         <v>120</v>
       </c>
       <c r="I16" s="5" t="s">
-        <v>138</v>
+        <v>137</v>
       </c>
       <c r="J16" s="3"/>
       <c r="K16" s="8">
@@ -1547,7 +1547,7 @@
         <v>120</v>
       </c>
       <c r="I17" s="5" t="s">
-        <v>139</v>
+        <v>138</v>
       </c>
       <c r="J17" s="3"/>
       <c r="K17" s="6">
@@ -1580,7 +1580,7 @@
         <v>120</v>
       </c>
       <c r="I18" s="3" t="s">
-        <v>140</v>
+        <v>139</v>
       </c>
       <c r="J18" s="3"/>
       <c r="K18" s="6">
@@ -1613,7 +1613,7 @@
         <v>120</v>
       </c>
       <c r="I19" s="3" t="s">
-        <v>141</v>
+        <v>140</v>
       </c>
       <c r="J19" s="3"/>
       <c r="K19" s="6">
@@ -1646,7 +1646,7 @@
         <v>120</v>
       </c>
       <c r="I20" s="3" t="s">
-        <v>142</v>
+        <v>141</v>
       </c>
       <c r="J20" s="3"/>
       <c r="K20" s="6">
@@ -1679,7 +1679,7 @@
         <v>120</v>
       </c>
       <c r="I21" s="5" t="s">
-        <v>143</v>
+        <v>142</v>
       </c>
       <c r="J21" s="3"/>
       <c r="K21" s="6">
@@ -1712,7 +1712,7 @@
         <v>120</v>
       </c>
       <c r="I22" s="5" t="s">
-        <v>149</v>
+        <v>148</v>
       </c>
       <c r="J22" s="3"/>
       <c r="K22" s="6">
@@ -1745,7 +1745,7 @@
         <v>120</v>
       </c>
       <c r="I23" s="5" t="s">
-        <v>149</v>
+        <v>148</v>
       </c>
       <c r="J23" s="3"/>
       <c r="K23" s="6">
@@ -1778,7 +1778,7 @@
         <v>120</v>
       </c>
       <c r="I24" s="5" t="s">
-        <v>151</v>
+        <v>150</v>
       </c>
       <c r="J24" s="3"/>
       <c r="K24" s="6">
@@ -1943,7 +1943,7 @@
         <v>120</v>
       </c>
       <c r="I29" s="5" t="s">
-        <v>143</v>
+        <v>142</v>
       </c>
       <c r="J29" s="3"/>
       <c r="K29" s="6">
@@ -1976,7 +1976,7 @@
         <v>120</v>
       </c>
       <c r="I30" s="5" t="s">
-        <v>150</v>
+        <v>149</v>
       </c>
       <c r="J30" s="3"/>
       <c r="K30" s="6">
@@ -2009,7 +2009,7 @@
         <v>120</v>
       </c>
       <c r="I31" s="5" t="s">
-        <v>152</v>
+        <v>151</v>
       </c>
       <c r="J31" s="3"/>
       <c r="K31" s="6">
@@ -2042,7 +2042,7 @@
         <v>120</v>
       </c>
       <c r="I32" s="5" t="s">
-        <v>149</v>
+        <v>148</v>
       </c>
       <c r="J32" s="3"/>
       <c r="K32" s="6">
@@ -2075,7 +2075,7 @@
         <v>120</v>
       </c>
       <c r="I33" s="5" t="s">
-        <v>149</v>
+        <v>148</v>
       </c>
       <c r="J33" s="3"/>
       <c r="K33" s="6">
@@ -2108,7 +2108,7 @@
         <v>120</v>
       </c>
       <c r="I34" s="5" t="s">
-        <v>154</v>
+        <v>153</v>
       </c>
       <c r="J34" s="3"/>
       <c r="K34" s="6">
@@ -2141,7 +2141,7 @@
         <v>120</v>
       </c>
       <c r="I35" s="5" t="s">
-        <v>155</v>
+        <v>154</v>
       </c>
       <c r="J35" s="3"/>
       <c r="K35" s="6">
@@ -2171,10 +2171,10 @@
         <v>100</v>
       </c>
       <c r="H36" s="3" t="s">
-        <v>130</v>
+        <v>129</v>
       </c>
       <c r="I36" s="5" t="s">
-        <v>144</v>
+        <v>143</v>
       </c>
       <c r="J36" s="3"/>
       <c r="K36" s="6">
@@ -2207,7 +2207,7 @@
         <v>120</v>
       </c>
       <c r="I37" s="5" t="s">
-        <v>143</v>
+        <v>142</v>
       </c>
       <c r="J37" s="3"/>
       <c r="K37" s="6">
@@ -2240,7 +2240,7 @@
         <v>123</v>
       </c>
       <c r="I38" s="5" t="s">
-        <v>144</v>
+        <v>143</v>
       </c>
       <c r="J38" s="3"/>
       <c r="K38" s="6">
@@ -2270,10 +2270,10 @@
         <v>97</v>
       </c>
       <c r="H39" s="3" t="s">
-        <v>158</v>
+        <v>157</v>
       </c>
       <c r="I39" s="5" t="s">
-        <v>145</v>
+        <v>144</v>
       </c>
       <c r="J39" s="3"/>
       <c r="K39" s="6">
@@ -2306,7 +2306,7 @@
         <v>120</v>
       </c>
       <c r="I40" s="5" t="s">
-        <v>144</v>
+        <v>143</v>
       </c>
       <c r="J40" s="3"/>
       <c r="K40" s="6">
@@ -2339,7 +2339,7 @@
         <v>120</v>
       </c>
       <c r="I41" s="5" t="s">
-        <v>148</v>
+        <v>147</v>
       </c>
       <c r="J41" s="3"/>
       <c r="K41" s="6">
@@ -2372,7 +2372,7 @@
         <v>120</v>
       </c>
       <c r="I42" s="5" t="s">
-        <v>148</v>
+        <v>147</v>
       </c>
       <c r="J42" s="3"/>
       <c r="K42" s="6">
@@ -2405,7 +2405,7 @@
         <v>123</v>
       </c>
       <c r="I43" s="5" t="s">
-        <v>144</v>
+        <v>143</v>
       </c>
       <c r="J43" s="3"/>
       <c r="K43" s="6">
@@ -2438,7 +2438,7 @@
         <v>120</v>
       </c>
       <c r="I44" s="5" t="s">
-        <v>143</v>
+        <v>142</v>
       </c>
       <c r="J44" s="3"/>
       <c r="K44" s="6">
@@ -2471,7 +2471,7 @@
         <v>120</v>
       </c>
       <c r="I45" s="5" t="s">
-        <v>144</v>
+        <v>143</v>
       </c>
       <c r="J45" s="3"/>
       <c r="K45" s="6">
@@ -2504,7 +2504,7 @@
         <v>120</v>
       </c>
       <c r="I46" s="5" t="s">
-        <v>159</v>
+        <v>158</v>
       </c>
       <c r="J46" s="3"/>
       <c r="K46" s="6">
@@ -2537,7 +2537,7 @@
         <v>120</v>
       </c>
       <c r="I47" s="5" t="s">
-        <v>144</v>
+        <v>143</v>
       </c>
       <c r="J47" s="3"/>
       <c r="K47" s="6">
@@ -2570,7 +2570,7 @@
         <v>120</v>
       </c>
       <c r="I48" s="5" t="s">
-        <v>163</v>
+        <v>162</v>
       </c>
       <c r="J48" s="3"/>
       <c r="K48" s="6">
@@ -2603,7 +2603,7 @@
         <v>120</v>
       </c>
       <c r="I49" s="5" t="s">
-        <v>144</v>
+        <v>143</v>
       </c>
       <c r="J49" s="3"/>
       <c r="K49" s="6">
@@ -2636,10 +2636,10 @@
         <v>120</v>
       </c>
       <c r="I50" s="5" t="s">
-        <v>162</v>
+        <v>161</v>
       </c>
       <c r="J50" s="3" t="s">
-        <v>165</v>
+        <v>164</v>
       </c>
       <c r="K50" s="6">
         <v>46311</v>
@@ -2671,10 +2671,10 @@
         <v>120</v>
       </c>
       <c r="I51" s="5" t="s">
-        <v>144</v>
+        <v>143</v>
       </c>
       <c r="J51" s="3" t="s">
-        <v>166</v>
+        <v>165</v>
       </c>
       <c r="K51" s="6">
         <v>46311</v>
@@ -2706,10 +2706,10 @@
         <v>120</v>
       </c>
       <c r="I52" s="5" t="s">
-        <v>144</v>
+        <v>143</v>
       </c>
       <c r="J52" s="3" t="s">
-        <v>166</v>
+        <v>165</v>
       </c>
       <c r="K52" s="6">
         <v>46311</v>
@@ -2742,7 +2742,7 @@
         <v>120</v>
       </c>
       <c r="I53" s="5" t="s">
-        <v>161</v>
+        <v>160</v>
       </c>
       <c r="J53" s="3"/>
       <c r="K53" s="6">
@@ -2775,7 +2775,7 @@
         <v>120</v>
       </c>
       <c r="I54" s="5" t="s">
-        <v>147</v>
+        <v>146</v>
       </c>
       <c r="J54" s="3"/>
       <c r="K54" s="6">
@@ -2808,7 +2808,7 @@
         <v>120</v>
       </c>
       <c r="I55" s="5" t="s">
-        <v>162</v>
+        <v>161</v>
       </c>
       <c r="J55" s="3"/>
       <c r="K55" s="6">
@@ -2838,10 +2838,10 @@
         <v>91</v>
       </c>
       <c r="H56" s="3" t="s">
-        <v>130</v>
+        <v>129</v>
       </c>
       <c r="I56" s="5" t="s">
-        <v>143</v>
+        <v>142</v>
       </c>
       <c r="J56" s="3"/>
       <c r="K56" s="6">
@@ -2871,10 +2871,10 @@
         <v>94</v>
       </c>
       <c r="H57" s="3" t="s">
-        <v>130</v>
+        <v>129</v>
       </c>
       <c r="I57" s="5" t="s">
-        <v>144</v>
+        <v>143</v>
       </c>
       <c r="J57" s="3"/>
       <c r="K57" s="6">
@@ -2907,7 +2907,7 @@
         <v>120</v>
       </c>
       <c r="I58" s="5" t="s">
-        <v>160</v>
+        <v>159</v>
       </c>
       <c r="J58" s="3"/>
       <c r="K58" s="6">
@@ -2940,7 +2940,7 @@
         <v>120</v>
       </c>
       <c r="I59" s="5" t="s">
-        <v>145</v>
+        <v>144</v>
       </c>
       <c r="J59" s="3"/>
       <c r="K59" s="6">
@@ -2973,7 +2973,7 @@
         <v>120</v>
       </c>
       <c r="I60" s="5" t="s">
-        <v>147</v>
+        <v>146</v>
       </c>
       <c r="J60" s="3"/>
       <c r="K60" s="6">
@@ -3006,7 +3006,7 @@
         <v>120</v>
       </c>
       <c r="I61" s="5" t="s">
-        <v>147</v>
+        <v>146</v>
       </c>
       <c r="J61" s="3"/>
       <c r="K61" s="6">
@@ -3039,7 +3039,7 @@
         <v>120</v>
       </c>
       <c r="I62" s="5" t="s">
-        <v>144</v>
+        <v>143</v>
       </c>
       <c r="J62" s="3"/>
       <c r="K62" s="6">
@@ -3069,7 +3069,7 @@
         <v>91</v>
       </c>
       <c r="H63" s="3" t="s">
-        <v>130</v>
+        <v>129</v>
       </c>
       <c r="I63" s="3" t="s">
         <v>91</v>
@@ -3102,10 +3102,10 @@
         <v>94</v>
       </c>
       <c r="H64" s="3" t="s">
-        <v>130</v>
+        <v>129</v>
       </c>
       <c r="I64" s="5" t="s">
-        <v>144</v>
+        <v>143</v>
       </c>
       <c r="J64" s="3"/>
       <c r="K64" s="6">
@@ -3171,7 +3171,7 @@
         <v>120</v>
       </c>
       <c r="I66" s="5" t="s">
-        <v>144</v>
+        <v>143</v>
       </c>
       <c r="J66" s="3"/>
       <c r="K66" s="6">
@@ -3204,7 +3204,7 @@
         <v>120</v>
       </c>
       <c r="I67" s="5" t="s">
-        <v>143</v>
+        <v>142</v>
       </c>
       <c r="J67" s="3"/>
       <c r="K67" s="6">
@@ -3237,7 +3237,7 @@
         <v>120</v>
       </c>
       <c r="I68" s="5" t="s">
-        <v>144</v>
+        <v>143</v>
       </c>
       <c r="J68" s="3"/>
       <c r="K68" s="6">
@@ -3270,7 +3270,7 @@
         <v>120</v>
       </c>
       <c r="I69" s="5" t="s">
-        <v>153</v>
+        <v>152</v>
       </c>
       <c r="J69" s="3"/>
       <c r="K69" s="6">
@@ -3303,7 +3303,7 @@
         <v>120</v>
       </c>
       <c r="I70" s="5" t="s">
-        <v>147</v>
+        <v>146</v>
       </c>
       <c r="J70" s="3"/>
       <c r="K70" s="6">
@@ -3336,7 +3336,7 @@
         <v>120</v>
       </c>
       <c r="I71" s="5" t="s">
-        <v>147</v>
+        <v>146</v>
       </c>
       <c r="J71" s="3"/>
       <c r="K71" s="6">
@@ -3369,7 +3369,7 @@
         <v>120</v>
       </c>
       <c r="I72" s="5" t="s">
-        <v>156</v>
+        <v>155</v>
       </c>
       <c r="J72" s="3"/>
       <c r="K72" s="6">
@@ -3402,7 +3402,7 @@
         <v>120</v>
       </c>
       <c r="I73" s="5" t="s">
-        <v>144</v>
+        <v>143</v>
       </c>
       <c r="J73" s="3"/>
       <c r="K73" s="6">
@@ -3435,7 +3435,7 @@
         <v>120</v>
       </c>
       <c r="I74" s="5" t="s">
-        <v>143</v>
+        <v>142</v>
       </c>
       <c r="J74" s="3"/>
       <c r="K74" s="6">
@@ -3468,7 +3468,7 @@
         <v>120</v>
       </c>
       <c r="I75" s="5" t="s">
-        <v>144</v>
+        <v>143</v>
       </c>
       <c r="J75" s="3"/>
       <c r="K75" s="6">
@@ -3501,7 +3501,7 @@
         <v>120</v>
       </c>
       <c r="I76" s="5" t="s">
-        <v>156</v>
+        <v>155</v>
       </c>
       <c r="J76" s="3"/>
       <c r="K76" s="6">
@@ -3534,7 +3534,7 @@
         <v>120</v>
       </c>
       <c r="I77" s="5" t="s">
-        <v>144</v>
+        <v>143</v>
       </c>
       <c r="J77" s="3"/>
       <c r="K77" s="6">
@@ -3567,7 +3567,7 @@
         <v>120</v>
       </c>
       <c r="I78" s="5" t="s">
-        <v>144</v>
+        <v>143</v>
       </c>
       <c r="J78" s="3"/>
       <c r="K78" s="6">
@@ -3600,7 +3600,7 @@
         <v>120</v>
       </c>
       <c r="I79" s="5" t="s">
-        <v>146</v>
+        <v>145</v>
       </c>
       <c r="J79" s="3"/>
       <c r="K79" s="6">
@@ -3633,7 +3633,7 @@
         <v>120</v>
       </c>
       <c r="I80" s="5" t="s">
-        <v>146</v>
+        <v>145</v>
       </c>
       <c r="J80" s="3"/>
       <c r="K80" s="6">
@@ -3666,7 +3666,7 @@
         <v>120</v>
       </c>
       <c r="I81" s="5" t="s">
-        <v>143</v>
+        <v>142</v>
       </c>
       <c r="J81" s="3"/>
       <c r="K81" s="6">
@@ -3699,7 +3699,7 @@
         <v>120</v>
       </c>
       <c r="I82" s="5" t="s">
-        <v>144</v>
+        <v>143</v>
       </c>
       <c r="J82" s="3"/>
       <c r="K82" s="6">
@@ -3732,7 +3732,7 @@
         <v>120</v>
       </c>
       <c r="I83" s="5" t="s">
-        <v>156</v>
+        <v>155</v>
       </c>
       <c r="J83" s="3"/>
       <c r="K83" s="6">
@@ -3765,7 +3765,7 @@
         <v>120</v>
       </c>
       <c r="I84" s="5" t="s">
-        <v>144</v>
+        <v>143</v>
       </c>
       <c r="J84" s="3"/>
       <c r="K84" s="6">
@@ -3798,7 +3798,7 @@
         <v>120</v>
       </c>
       <c r="I85" s="5" t="s">
-        <v>143</v>
+        <v>142</v>
       </c>
       <c r="J85" s="3"/>
       <c r="K85" s="6">
@@ -3831,7 +3831,7 @@
         <v>120</v>
       </c>
       <c r="I86" s="5" t="s">
-        <v>144</v>
+        <v>143</v>
       </c>
       <c r="J86" s="3"/>
       <c r="K86" s="6">
@@ -3864,7 +3864,7 @@
         <v>120</v>
       </c>
       <c r="I87" s="5" t="s">
-        <v>144</v>
+        <v>143</v>
       </c>
       <c r="J87" s="3"/>
       <c r="K87" s="6">
@@ -3897,7 +3897,7 @@
         <v>120</v>
       </c>
       <c r="I88" s="5" t="s">
-        <v>153</v>
+        <v>152</v>
       </c>
       <c r="J88" s="3"/>
       <c r="K88" s="6">
@@ -3930,7 +3930,7 @@
         <v>120</v>
       </c>
       <c r="I89" s="5" t="s">
-        <v>147</v>
+        <v>146</v>
       </c>
       <c r="J89" s="3"/>
       <c r="K89" s="6">
@@ -3996,7 +3996,7 @@
         <v>120</v>
       </c>
       <c r="I91" s="5" t="s">
-        <v>156</v>
+        <v>155</v>
       </c>
       <c r="J91" s="3"/>
       <c r="K91" s="6">
@@ -4029,7 +4029,7 @@
         <v>120</v>
       </c>
       <c r="I92" s="5" t="s">
-        <v>144</v>
+        <v>143</v>
       </c>
       <c r="J92" s="3"/>
       <c r="K92" s="6">
@@ -4062,7 +4062,7 @@
         <v>120</v>
       </c>
       <c r="I93" s="5" t="s">
-        <v>143</v>
+        <v>142</v>
       </c>
       <c r="J93" s="3"/>
       <c r="K93" s="6">
@@ -4095,7 +4095,7 @@
         <v>120</v>
       </c>
       <c r="I94" s="5" t="s">
-        <v>144</v>
+        <v>143</v>
       </c>
       <c r="J94" s="3"/>
       <c r="K94" s="6">
@@ -4128,7 +4128,7 @@
         <v>123</v>
       </c>
       <c r="I95" s="5" t="s">
-        <v>157</v>
+        <v>156</v>
       </c>
       <c r="J95" s="3"/>
       <c r="K95" s="6">
@@ -4161,7 +4161,7 @@
         <v>120</v>
       </c>
       <c r="I96" s="5" t="s">
-        <v>144</v>
+        <v>143</v>
       </c>
       <c r="J96" s="3"/>
       <c r="K96" s="6">

</xml_diff>